<commit_message>
Publish LeeValley_2015_WCH, LeeValley_2019_WC, LeeValley_2023_WCH, LiptovskyMikulas_2015_WC
</commit_message>
<xml_diff>
--- a/events/LeeValley_2019_WC/LeeValley_2019_WC_start.xlsx
+++ b/events/LeeValley_2019_WC/LeeValley_2019_WC_start.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W587"/>
+  <dimension ref="A1:AC587"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -519,17 +519,47 @@
       </c>
       <c r="U1" t="inlineStr">
         <is>
+          <t>Name4</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>Name5</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>Name6</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
           <t>ICF_ID1</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>ICF_ID2</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>ICF_ID3</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>ICF_ID4</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>ICF_ID5</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>ICF_ID6</t>
         </is>
       </c>
     </row>
@@ -787,7 +817,7 @@
           <t>XU Yongzhao</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr">
+      <c r="X6" t="inlineStr">
         <is>
           <t>69446</t>
         </is>
@@ -845,7 +875,7 @@
           <t>ZOU Weijian</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr">
+      <c r="X7" t="inlineStr">
         <is>
           <t>94208</t>
         </is>
@@ -903,7 +933,7 @@
           <t>HUANG Fa</t>
         </is>
       </c>
-      <c r="U8" t="inlineStr">
+      <c r="X8" t="inlineStr">
         <is>
           <t>87703</t>
         </is>
@@ -961,7 +991,7 @@
           <t>KOTOV Pavel</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr">
+      <c r="X9" t="inlineStr">
         <is>
           <t>66761</t>
         </is>
@@ -1019,7 +1049,7 @@
           <t>CHAKIR Issam</t>
         </is>
       </c>
-      <c r="U10" t="inlineStr">
+      <c r="X10" t="inlineStr">
         <is>
           <t>75631</t>
         </is>
@@ -1077,7 +1107,7 @@
           <t>CARVALHO Jose</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr">
+      <c r="X11" t="inlineStr">
         <is>
           <t>35486</t>
         </is>
@@ -1135,7 +1165,7 @@
           <t>SARAMANDIF Terence</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr">
+      <c r="X12" t="inlineStr">
         <is>
           <t>79340</t>
         </is>
@@ -1193,7 +1223,7 @@
           <t>LONG Tren</t>
         </is>
       </c>
-      <c r="U13" t="inlineStr">
+      <c r="X13" t="inlineStr">
         <is>
           <t>57124</t>
         </is>
@@ -1251,7 +1281,7 @@
           <t>HEGER Vojtech</t>
         </is>
       </c>
-      <c r="U14" t="inlineStr">
+      <c r="X14" t="inlineStr">
         <is>
           <t>68872</t>
         </is>
@@ -1309,7 +1339,7 @@
           <t>WASHER Patrick</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr">
+      <c r="X15" t="inlineStr">
         <is>
           <t>42081</t>
         </is>
@@ -1367,7 +1397,7 @@
           <t>HENDRICK Robert</t>
         </is>
       </c>
-      <c r="U16" t="inlineStr">
+      <c r="X16" t="inlineStr">
         <is>
           <t>43002</t>
         </is>
@@ -1425,7 +1455,7 @@
           <t>GIBB Benjamin</t>
         </is>
       </c>
-      <c r="U17" t="inlineStr">
+      <c r="X17" t="inlineStr">
         <is>
           <t>36711</t>
         </is>
@@ -1483,7 +1513,7 @@
           <t>LOWTHER Steven</t>
         </is>
       </c>
-      <c r="U18" t="inlineStr">
+      <c r="X18" t="inlineStr">
         <is>
           <t>44811</t>
         </is>
@@ -1541,7 +1571,7 @@
           <t>COCHRANE Jake</t>
         </is>
       </c>
-      <c r="U19" t="inlineStr">
+      <c r="X19" t="inlineStr">
         <is>
           <t>60124</t>
         </is>
@@ -1599,7 +1629,7 @@
           <t>KHRAMTSOV Dmitrii</t>
         </is>
       </c>
-      <c r="U20" t="inlineStr">
+      <c r="X20" t="inlineStr">
         <is>
           <t>66768</t>
         </is>
@@ -1657,7 +1687,7 @@
           <t>BOURHIS Jean Pierre</t>
         </is>
       </c>
-      <c r="U21" t="inlineStr">
+      <c r="X21" t="inlineStr">
         <is>
           <t>36968</t>
         </is>
@@ -1715,7 +1745,7 @@
           <t>BOURHIS Yves</t>
         </is>
       </c>
-      <c r="U22" t="inlineStr">
+      <c r="X22" t="inlineStr">
         <is>
           <t>63237</t>
         </is>
@@ -1773,7 +1803,7 @@
           <t>BORGES Felipe</t>
         </is>
       </c>
-      <c r="U23" t="inlineStr">
+      <c r="X23" t="inlineStr">
         <is>
           <t>38012</t>
         </is>
@@ -1831,7 +1861,7 @@
           <t>BREUER Florian</t>
         </is>
       </c>
-      <c r="U24" t="inlineStr">
+      <c r="X24" t="inlineStr">
         <is>
           <t>39171</t>
         </is>
@@ -1889,7 +1919,7 @@
           <t>SZTUBA Igor</t>
         </is>
       </c>
-      <c r="U25" t="inlineStr">
+      <c r="X25" t="inlineStr">
         <is>
           <t>35087</t>
         </is>
@@ -1947,7 +1977,7 @@
           <t>LOKKEN Zachary</t>
         </is>
       </c>
-      <c r="U26" t="inlineStr">
+      <c r="X26" t="inlineStr">
         <is>
           <t>35069</t>
         </is>
@@ -2005,7 +2035,7 @@
           <t>SMEDLEY Cameron</t>
         </is>
       </c>
-      <c r="U27" t="inlineStr">
+      <c r="X27" t="inlineStr">
         <is>
           <t>35543</t>
         </is>
@@ -2063,7 +2093,7 @@
           <t>JEGOU Liam</t>
         </is>
       </c>
-      <c r="U28" t="inlineStr">
+      <c r="X28" t="inlineStr">
         <is>
           <t>35820</t>
         </is>
@@ -2121,7 +2151,7 @@
           <t>RAK Tomas</t>
         </is>
       </c>
-      <c r="U29" t="inlineStr">
+      <c r="X29" t="inlineStr">
         <is>
           <t>35056</t>
         </is>
@@ -2179,7 +2209,7 @@
           <t>WATKINS Daniel</t>
         </is>
       </c>
-      <c r="U30" t="inlineStr">
+      <c r="X30" t="inlineStr">
         <is>
           <t>38430</t>
         </is>
@@ -2237,7 +2267,7 @@
           <t>SZTUBA Kacper</t>
         </is>
       </c>
-      <c r="U31" t="inlineStr">
+      <c r="X31" t="inlineStr">
         <is>
           <t>53636</t>
         </is>
@@ -2295,7 +2325,7 @@
           <t>MARINIC Matija</t>
         </is>
       </c>
-      <c r="U32" t="inlineStr">
+      <c r="X32" t="inlineStr">
         <is>
           <t>35595</t>
         </is>
@@ -2353,7 +2383,7 @@
           <t>SETKIN Kirill</t>
         </is>
       </c>
-      <c r="U33" t="inlineStr">
+      <c r="X33" t="inlineStr">
         <is>
           <t>35457</t>
         </is>
@@ -2411,7 +2441,7 @@
           <t>CIPRESSI Stefano</t>
         </is>
       </c>
-      <c r="U34" t="inlineStr">
+      <c r="X34" t="inlineStr">
         <is>
           <t>35495</t>
         </is>
@@ -2469,7 +2499,7 @@
           <t>BORROWS Ian</t>
         </is>
       </c>
-      <c r="U35" t="inlineStr">
+      <c r="X35" t="inlineStr">
         <is>
           <t>36534</t>
         </is>
@@ -2527,7 +2557,7 @@
           <t>KOECHLIN Thomas</t>
         </is>
       </c>
-      <c r="U36" t="inlineStr">
+      <c r="X36" t="inlineStr">
         <is>
           <t>35419</t>
         </is>
@@ -2585,7 +2615,7 @@
           <t>TRAVE Miquel</t>
         </is>
       </c>
-      <c r="U37" t="inlineStr">
+      <c r="X37" t="inlineStr">
         <is>
           <t>68998</t>
         </is>
@@ -2643,7 +2673,7 @@
           <t>EICHFELD Casey</t>
         </is>
       </c>
-      <c r="U38" t="inlineStr">
+      <c r="X38" t="inlineStr">
         <is>
           <t>35067</t>
         </is>
@@ -2701,7 +2731,7 @@
           <t>COLAZINGARI Roberto</t>
         </is>
       </c>
-      <c r="U39" t="inlineStr">
+      <c r="X39" t="inlineStr">
         <is>
           <t>35223</t>
         </is>
@@ -2759,7 +2789,7 @@
           <t>JOLY Cedric</t>
         </is>
       </c>
-      <c r="U40" t="inlineStr">
+      <c r="X40" t="inlineStr">
         <is>
           <t>35681</t>
         </is>
@@ -2817,7 +2847,7 @@
           <t>ELOSEGI Ander</t>
         </is>
       </c>
-      <c r="U41" t="inlineStr">
+      <c r="X41" t="inlineStr">
         <is>
           <t>35785</t>
         </is>
@@ -2875,7 +2905,7 @@
           <t>BERCIC Anze</t>
         </is>
       </c>
-      <c r="U42" t="inlineStr">
+      <c r="X42" t="inlineStr">
         <is>
           <t>36253</t>
         </is>
@@ -2933,7 +2963,7 @@
           <t>BURGESS Adam</t>
         </is>
       </c>
-      <c r="U43" t="inlineStr">
+      <c r="X43" t="inlineStr">
         <is>
           <t>35647</t>
         </is>
@@ -2991,7 +3021,7 @@
           <t>FLORENCE David</t>
         </is>
       </c>
-      <c r="U44" t="inlineStr">
+      <c r="X44" t="inlineStr">
         <is>
           <t>35634</t>
         </is>
@@ -3049,7 +3079,7 @@
           <t>HEDWIG Grzegorz</t>
         </is>
       </c>
-      <c r="U45" t="inlineStr">
+      <c r="X45" t="inlineStr">
         <is>
           <t>35465</t>
         </is>
@@ -3107,7 +3137,7 @@
           <t>IVALDI Raffaello</t>
         </is>
       </c>
-      <c r="U46" t="inlineStr">
+      <c r="X46" t="inlineStr">
         <is>
           <t>35227</t>
         </is>
@@ -3165,7 +3195,7 @@
           <t>ROHAN Lukas</t>
         </is>
       </c>
-      <c r="U47" t="inlineStr">
+      <c r="X47" t="inlineStr">
         <is>
           <t>36114</t>
         </is>
@@ -3223,7 +3253,7 @@
           <t>THOMAS Martin</t>
         </is>
       </c>
-      <c r="U48" t="inlineStr">
+      <c r="X48" t="inlineStr">
         <is>
           <t>35412</t>
         </is>
@@ -3281,7 +3311,7 @@
           <t>GARGAUD CHANUT Denis</t>
         </is>
       </c>
-      <c r="U49" t="inlineStr">
+      <c r="X49" t="inlineStr">
         <is>
           <t>35177</t>
         </is>
@@ -3339,7 +3369,7 @@
           <t>MARTIKAN Michal</t>
         </is>
       </c>
-      <c r="U50" t="inlineStr">
+      <c r="X50" t="inlineStr">
         <is>
           <t>35365</t>
         </is>
@@ -3397,7 +3427,7 @@
           <t>BOZIC Luka</t>
         </is>
       </c>
-      <c r="U51" t="inlineStr">
+      <c r="X51" t="inlineStr">
         <is>
           <t>36269</t>
         </is>
@@ -3455,7 +3485,7 @@
           <t>WESTLEY Ryan</t>
         </is>
       </c>
-      <c r="U52" t="inlineStr">
+      <c r="X52" t="inlineStr">
         <is>
           <t>35651</t>
         </is>
@@ -3513,7 +3543,7 @@
           <t>BENUS Matej</t>
         </is>
       </c>
-      <c r="U53" t="inlineStr">
+      <c r="X53" t="inlineStr">
         <is>
           <t>35353</t>
         </is>
@@ -3571,7 +3601,7 @@
           <t>ANTON Franz</t>
         </is>
       </c>
-      <c r="U54" t="inlineStr">
+      <c r="X54" t="inlineStr">
         <is>
           <t>35137</t>
         </is>
@@ -3629,7 +3659,7 @@
           <t>SAVSEK Benjamin</t>
         </is>
       </c>
-      <c r="U55" t="inlineStr">
+      <c r="X55" t="inlineStr">
         <is>
           <t>36218</t>
         </is>
@@ -3687,7 +3717,7 @@
           <t>SLAFKOVSKY Alexander</t>
         </is>
       </c>
-      <c r="U56" t="inlineStr">
+      <c r="X56" t="inlineStr">
         <is>
           <t>35129</t>
         </is>
@@ -3745,7 +3775,7 @@
           <t>TASIADIS Sideris</t>
         </is>
       </c>
-      <c r="U57" t="inlineStr">
+      <c r="X57" t="inlineStr">
         <is>
           <t>35135</t>
         </is>
@@ -3803,7 +3833,7 @@
           <t>TOROK Luca</t>
         </is>
       </c>
-      <c r="U58" t="inlineStr">
+      <c r="X58" t="inlineStr">
         <is>
           <t>94043</t>
         </is>
@@ -3861,7 +3891,7 @@
           <t>NICHOLAS Ella</t>
         </is>
       </c>
-      <c r="U59" t="inlineStr">
+      <c r="X59" t="inlineStr">
         <is>
           <t>36591</t>
         </is>
@@ -3919,7 +3949,7 @@
           <t>SORRIBES Laia</t>
         </is>
       </c>
-      <c r="U60" t="inlineStr">
+      <c r="X60" t="inlineStr">
         <is>
           <t>68822</t>
         </is>
@@ -3977,7 +4007,7 @@
           <t>NICHOLAS Jane</t>
         </is>
       </c>
-      <c r="U61" t="inlineStr">
+      <c r="X61" t="inlineStr">
         <is>
           <t>93757</t>
         </is>
@@ -4035,7 +4065,7 @@
           <t>THOMAS Hannah</t>
         </is>
       </c>
-      <c r="U62" t="inlineStr">
+      <c r="X62" t="inlineStr">
         <is>
           <t>85758</t>
         </is>
@@ -4093,7 +4123,7 @@
           <t>XU Yanru</t>
         </is>
       </c>
-      <c r="U63" t="inlineStr">
+      <c r="X63" t="inlineStr">
         <is>
           <t>63801</t>
         </is>
@@ -4151,7 +4181,7 @@
           <t>RANDLE Kensa</t>
         </is>
       </c>
-      <c r="U64" t="inlineStr">
+      <c r="X64" t="inlineStr">
         <is>
           <t>51859</t>
         </is>
@@ -4209,7 +4239,7 @@
           <t>BETTERIDGE Lois</t>
         </is>
       </c>
-      <c r="U65" t="inlineStr">
+      <c r="X65" t="inlineStr">
         <is>
           <t>60078</t>
         </is>
@@ -4267,7 +4297,7 @@
           <t>MITASIKOVA Monika</t>
         </is>
       </c>
-      <c r="U66" t="inlineStr">
+      <c r="X66" t="inlineStr">
         <is>
           <t>75445</t>
         </is>
@@ -4325,7 +4355,7 @@
           <t>DONNELLY Sage</t>
         </is>
       </c>
-      <c r="U67" t="inlineStr">
+      <c r="X67" t="inlineStr">
         <is>
           <t>60119</t>
         </is>
@@ -4383,7 +4413,7 @@
           <t>MINAZOVA Alsu</t>
         </is>
       </c>
-      <c r="U68" t="inlineStr">
+      <c r="X68" t="inlineStr">
         <is>
           <t>53314</t>
         </is>
@@ -4441,7 +4471,7 @@
           <t>NEE Ashley</t>
         </is>
       </c>
-      <c r="U69" t="inlineStr">
+      <c r="X69" t="inlineStr">
         <is>
           <t>36363</t>
         </is>
@@ -4499,7 +4529,7 @@
           <t>VILARRUBLA Nuria</t>
         </is>
       </c>
-      <c r="U70" t="inlineStr">
+      <c r="X70" t="inlineStr">
         <is>
           <t>35746</t>
         </is>
@@ -4557,7 +4587,7 @@
           <t>APEL Elena</t>
         </is>
       </c>
-      <c r="U71" t="inlineStr">
+      <c r="X71" t="inlineStr">
         <is>
           <t>51837</t>
         </is>
@@ -4615,7 +4645,7 @@
           <t>FOX Noemie</t>
         </is>
       </c>
-      <c r="U72" t="inlineStr">
+      <c r="X72" t="inlineStr">
         <is>
           <t>44812</t>
         </is>
@@ -4673,7 +4703,7 @@
           <t>NOVAK Ajda</t>
         </is>
       </c>
-      <c r="U73" t="inlineStr">
+      <c r="X73" t="inlineStr">
         <is>
           <t>39079</t>
         </is>
@@ -4731,7 +4761,7 @@
           <t>DORIA VILARRUBLA Monica</t>
         </is>
       </c>
-      <c r="U74" t="inlineStr">
+      <c r="X74" t="inlineStr">
         <is>
           <t>53051</t>
         </is>
@@ -4789,7 +4819,7 @@
           <t>LI Tong</t>
         </is>
       </c>
-      <c r="U75" t="inlineStr">
+      <c r="X75" t="inlineStr">
         <is>
           <t>52023</t>
         </is>
@@ -4847,7 +4877,7 @@
           <t>MINTALOVA Eliska</t>
         </is>
       </c>
-      <c r="U76" t="inlineStr">
+      <c r="X76" t="inlineStr">
         <is>
           <t>56169</t>
         </is>
@@ -4905,7 +4935,7 @@
           <t>KALISKA Elena</t>
         </is>
       </c>
-      <c r="U77" t="inlineStr">
+      <c r="X77" t="inlineStr">
         <is>
           <t>35366</t>
         </is>
@@ -4963,7 +4993,7 @@
           <t>PEROVA Ekaterina</t>
         </is>
       </c>
-      <c r="U78" t="inlineStr">
+      <c r="X78" t="inlineStr">
         <is>
           <t>35131</t>
         </is>
@@ -5021,7 +5051,7 @@
           <t>VOJTOVA Veronika</t>
         </is>
       </c>
-      <c r="U79" t="inlineStr">
+      <c r="X79" t="inlineStr">
         <is>
           <t>35945</t>
         </is>
@@ -5079,7 +5109,7 @@
           <t>HILGERTOVA Amalie</t>
         </is>
       </c>
-      <c r="U80" t="inlineStr">
+      <c r="X80" t="inlineStr">
         <is>
           <t>36113</t>
         </is>
@@ -5137,7 +5167,7 @@
           <t>LAFONT Marie-Zelia</t>
         </is>
       </c>
-      <c r="U81" t="inlineStr">
+      <c r="X81" t="inlineStr">
         <is>
           <t>35374</t>
         </is>
@@ -5195,7 +5225,7 @@
           <t>ZWOLINSKA Klaudia</t>
         </is>
       </c>
-      <c r="U82" t="inlineStr">
+      <c r="X82" t="inlineStr">
         <is>
           <t>42027</t>
         </is>
@@ -5253,7 +5283,7 @@
           <t>WOODS Kimberley</t>
         </is>
       </c>
-      <c r="U83" t="inlineStr">
+      <c r="X83" t="inlineStr">
         <is>
           <t>35650</t>
         </is>
@@ -5311,7 +5341,7 @@
           <t>LAWRENCE Rosalyn</t>
         </is>
       </c>
-      <c r="U84" t="inlineStr">
+      <c r="X84" t="inlineStr">
         <is>
           <t>36531</t>
         </is>
@@ -5369,7 +5399,7 @@
           <t>JONES Luuka</t>
         </is>
       </c>
-      <c r="U85" t="inlineStr">
+      <c r="X85" t="inlineStr">
         <is>
           <t>36657</t>
         </is>
@@ -5427,7 +5457,7 @@
           <t>BAUDU Lucie</t>
         </is>
       </c>
-      <c r="U86" t="inlineStr">
+      <c r="X86" t="inlineStr">
         <is>
           <t>35669</t>
         </is>
@@ -5485,7 +5515,7 @@
           <t>KHARITONOVA Marta</t>
         </is>
       </c>
-      <c r="U87" t="inlineStr">
+      <c r="X87" t="inlineStr">
         <is>
           <t>35257</t>
         </is>
@@ -5543,7 +5573,7 @@
           <t>PACIERPNIK Natalia</t>
         </is>
       </c>
-      <c r="U88" t="inlineStr">
+      <c r="X88" t="inlineStr">
         <is>
           <t>35077</t>
         </is>
@@ -5601,7 +5631,7 @@
           <t>WOLFFHARDT Viktoria</t>
         </is>
       </c>
-      <c r="U89" t="inlineStr">
+      <c r="X89" t="inlineStr">
         <is>
           <t>35303</t>
         </is>
@@ -5659,7 +5689,7 @@
           <t>SATILA Ana</t>
         </is>
       </c>
-      <c r="U90" t="inlineStr">
+      <c r="X90" t="inlineStr">
         <is>
           <t>35327</t>
         </is>
@@ -5717,7 +5747,7 @@
           <t>PENNIE Fiona</t>
         </is>
       </c>
-      <c r="U91" t="inlineStr">
+      <c r="X91" t="inlineStr">
         <is>
           <t>35638</t>
         </is>
@@ -5775,7 +5805,7 @@
           <t>KUDEJOVA Katerina</t>
         </is>
       </c>
-      <c r="U92" t="inlineStr">
+      <c r="X92" t="inlineStr">
         <is>
           <t>35034</t>
         </is>
@@ -5833,7 +5863,7 @@
           <t>SCHORNBERG Jasmin</t>
         </is>
       </c>
-      <c r="U93" t="inlineStr">
+      <c r="X93" t="inlineStr">
         <is>
           <t>35206</t>
         </is>
@@ -5891,7 +5921,7 @@
           <t>TERCELJ Eva</t>
         </is>
       </c>
-      <c r="U94" t="inlineStr">
+      <c r="X94" t="inlineStr">
         <is>
           <t>36263</t>
         </is>
@@ -5949,7 +5979,7 @@
           <t>HORN Stefanie</t>
         </is>
       </c>
-      <c r="U95" t="inlineStr">
+      <c r="X95" t="inlineStr">
         <is>
           <t>38417</t>
         </is>
@@ -6007,7 +6037,7 @@
           <t>DUKATOVA Jana</t>
         </is>
       </c>
-      <c r="U96" t="inlineStr">
+      <c r="X96" t="inlineStr">
         <is>
           <t>35354</t>
         </is>
@@ -6065,7 +6095,7 @@
           <t>PRIGENT Camille</t>
         </is>
       </c>
-      <c r="U97" t="inlineStr">
+      <c r="X97" t="inlineStr">
         <is>
           <t>41566</t>
         </is>
@@ -6123,7 +6153,7 @@
           <t>FRANKLIN Mallory</t>
         </is>
       </c>
-      <c r="U98" t="inlineStr">
+      <c r="X98" t="inlineStr">
         <is>
           <t>35615</t>
         </is>
@@ -6181,7 +6211,7 @@
           <t>KUHNLE Corinna</t>
         </is>
       </c>
-      <c r="U99" t="inlineStr">
+      <c r="X99" t="inlineStr">
         <is>
           <t>35282</t>
         </is>
@@ -6239,7 +6269,7 @@
           <t>KRAGELJ Ursa</t>
         </is>
       </c>
-      <c r="U100" t="inlineStr">
+      <c r="X100" t="inlineStr">
         <is>
           <t>36264</t>
         </is>
@@ -6297,7 +6327,7 @@
           <t>CHOURRAUT Maialen</t>
         </is>
       </c>
-      <c r="U101" t="inlineStr">
+      <c r="X101" t="inlineStr">
         <is>
           <t>35787</t>
         </is>
@@ -6355,7 +6385,7 @@
           <t>FUNK Ricarda</t>
         </is>
       </c>
-      <c r="U102" t="inlineStr">
+      <c r="X102" t="inlineStr">
         <is>
           <t>35122</t>
         </is>
@@ -6413,7 +6443,7 @@
           <t>FOX Jessica</t>
         </is>
       </c>
-      <c r="U103" t="inlineStr">
+      <c r="X103" t="inlineStr">
         <is>
           <t>36526</t>
         </is>
@@ -6471,7 +6501,7 @@
           <t>XU Yongzhao</t>
         </is>
       </c>
-      <c r="U104" t="inlineStr">
+      <c r="X104" t="inlineStr">
         <is>
           <t>69446</t>
         </is>
@@ -6529,7 +6559,7 @@
           <t>ZOU Weijian</t>
         </is>
       </c>
-      <c r="U105" t="inlineStr">
+      <c r="X105" t="inlineStr">
         <is>
           <t>94208</t>
         </is>
@@ -6587,7 +6617,7 @@
           <t>HUANG Fa</t>
         </is>
       </c>
-      <c r="U106" t="inlineStr">
+      <c r="X106" t="inlineStr">
         <is>
           <t>87703</t>
         </is>
@@ -6645,7 +6675,7 @@
           <t>KOTOV Pavel</t>
         </is>
       </c>
-      <c r="U107" t="inlineStr">
+      <c r="X107" t="inlineStr">
         <is>
           <t>66761</t>
         </is>
@@ -6703,7 +6733,7 @@
           <t>CHAKIR Issam</t>
         </is>
       </c>
-      <c r="U108" t="inlineStr">
+      <c r="X108" t="inlineStr">
         <is>
           <t>75631</t>
         </is>
@@ -6761,7 +6791,7 @@
           <t>CARVALHO Jose</t>
         </is>
       </c>
-      <c r="U109" t="inlineStr">
+      <c r="X109" t="inlineStr">
         <is>
           <t>35486</t>
         </is>
@@ -6819,7 +6849,7 @@
           <t>SARAMANDIF Terence</t>
         </is>
       </c>
-      <c r="U110" t="inlineStr">
+      <c r="X110" t="inlineStr">
         <is>
           <t>79340</t>
         </is>
@@ -6877,7 +6907,7 @@
           <t>LONG Tren</t>
         </is>
       </c>
-      <c r="U111" t="inlineStr">
+      <c r="X111" t="inlineStr">
         <is>
           <t>57124</t>
         </is>
@@ -6935,7 +6965,7 @@
           <t>HEGER Vojtech</t>
         </is>
       </c>
-      <c r="U112" t="inlineStr">
+      <c r="X112" t="inlineStr">
         <is>
           <t>68872</t>
         </is>
@@ -6993,7 +7023,7 @@
           <t>WASHER Patrick</t>
         </is>
       </c>
-      <c r="U113" t="inlineStr">
+      <c r="X113" t="inlineStr">
         <is>
           <t>42081</t>
         </is>
@@ -7051,7 +7081,7 @@
           <t>HENDRICK Robert</t>
         </is>
       </c>
-      <c r="U114" t="inlineStr">
+      <c r="X114" t="inlineStr">
         <is>
           <t>43002</t>
         </is>
@@ -7109,7 +7139,7 @@
           <t>GIBB Benjamin</t>
         </is>
       </c>
-      <c r="U115" t="inlineStr">
+      <c r="X115" t="inlineStr">
         <is>
           <t>36711</t>
         </is>
@@ -7167,7 +7197,7 @@
           <t>LOWTHER Steven</t>
         </is>
       </c>
-      <c r="U116" t="inlineStr">
+      <c r="X116" t="inlineStr">
         <is>
           <t>44811</t>
         </is>
@@ -7225,7 +7255,7 @@
           <t>COCHRANE Jake</t>
         </is>
       </c>
-      <c r="U117" t="inlineStr">
+      <c r="X117" t="inlineStr">
         <is>
           <t>60124</t>
         </is>
@@ -7283,7 +7313,7 @@
           <t>KHRAMTSOV Dmitrii</t>
         </is>
       </c>
-      <c r="U118" t="inlineStr">
+      <c r="X118" t="inlineStr">
         <is>
           <t>66768</t>
         </is>
@@ -7341,7 +7371,7 @@
           <t>BOURHIS Yves</t>
         </is>
       </c>
-      <c r="U119" t="inlineStr">
+      <c r="X119" t="inlineStr">
         <is>
           <t>63237</t>
         </is>
@@ -7399,7 +7429,7 @@
           <t>BORGES Felipe</t>
         </is>
       </c>
-      <c r="U120" t="inlineStr">
+      <c r="X120" t="inlineStr">
         <is>
           <t>38012</t>
         </is>
@@ -7457,7 +7487,7 @@
           <t>BREUER Florian</t>
         </is>
       </c>
-      <c r="U121" t="inlineStr">
+      <c r="X121" t="inlineStr">
         <is>
           <t>39171</t>
         </is>
@@ -7515,7 +7545,7 @@
           <t>SZTUBA Igor</t>
         </is>
       </c>
-      <c r="U122" t="inlineStr">
+      <c r="X122" t="inlineStr">
         <is>
           <t>35087</t>
         </is>
@@ -7573,7 +7603,7 @@
           <t>LOKKEN Zachary</t>
         </is>
       </c>
-      <c r="U123" t="inlineStr">
+      <c r="X123" t="inlineStr">
         <is>
           <t>35069</t>
         </is>
@@ -7631,7 +7661,7 @@
           <t>JEGOU Liam</t>
         </is>
       </c>
-      <c r="U124" t="inlineStr">
+      <c r="X124" t="inlineStr">
         <is>
           <t>35820</t>
         </is>
@@ -7689,7 +7719,7 @@
           <t>RAK Tomas</t>
         </is>
       </c>
-      <c r="U125" t="inlineStr">
+      <c r="X125" t="inlineStr">
         <is>
           <t>35056</t>
         </is>
@@ -7747,7 +7777,7 @@
           <t>WATKINS Daniel</t>
         </is>
       </c>
-      <c r="U126" t="inlineStr">
+      <c r="X126" t="inlineStr">
         <is>
           <t>38430</t>
         </is>
@@ -7805,7 +7835,7 @@
           <t>MARINIC Matija</t>
         </is>
       </c>
-      <c r="U127" t="inlineStr">
+      <c r="X127" t="inlineStr">
         <is>
           <t>35595</t>
         </is>
@@ -7863,7 +7893,7 @@
           <t>CIPRESSI Stefano</t>
         </is>
       </c>
-      <c r="U128" t="inlineStr">
+      <c r="X128" t="inlineStr">
         <is>
           <t>35495</t>
         </is>
@@ -7921,7 +7951,7 @@
           <t>BORROWS Ian</t>
         </is>
       </c>
-      <c r="U129" t="inlineStr">
+      <c r="X129" t="inlineStr">
         <is>
           <t>36534</t>
         </is>
@@ -7979,7 +8009,7 @@
           <t>TRAVE Miquel</t>
         </is>
       </c>
-      <c r="U130" t="inlineStr">
+      <c r="X130" t="inlineStr">
         <is>
           <t>68998</t>
         </is>
@@ -8037,7 +8067,7 @@
           <t>EICHFELD Casey</t>
         </is>
       </c>
-      <c r="U131" t="inlineStr">
+      <c r="X131" t="inlineStr">
         <is>
           <t>35067</t>
         </is>
@@ -8095,7 +8125,7 @@
           <t>JOLY Cedric</t>
         </is>
       </c>
-      <c r="U132" t="inlineStr">
+      <c r="X132" t="inlineStr">
         <is>
           <t>35681</t>
         </is>
@@ -8153,7 +8183,7 @@
           <t>BERCIC Anze</t>
         </is>
       </c>
-      <c r="U133" t="inlineStr">
+      <c r="X133" t="inlineStr">
         <is>
           <t>36253</t>
         </is>
@@ -8211,7 +8241,7 @@
           <t>HEDWIG Grzegorz</t>
         </is>
       </c>
-      <c r="U134" t="inlineStr">
+      <c r="X134" t="inlineStr">
         <is>
           <t>35465</t>
         </is>
@@ -8269,7 +8299,7 @@
           <t>IVALDI Raffaello</t>
         </is>
       </c>
-      <c r="U135" t="inlineStr">
+      <c r="X135" t="inlineStr">
         <is>
           <t>35227</t>
         </is>
@@ -8327,7 +8357,7 @@
           <t>TOROK Luca</t>
         </is>
       </c>
-      <c r="U136" t="inlineStr">
+      <c r="X136" t="inlineStr">
         <is>
           <t>94043</t>
         </is>
@@ -8385,7 +8415,7 @@
           <t>NICHOLAS Ella</t>
         </is>
       </c>
-      <c r="U137" t="inlineStr">
+      <c r="X137" t="inlineStr">
         <is>
           <t>36591</t>
         </is>
@@ -8443,7 +8473,7 @@
           <t>SORRIBES Laia</t>
         </is>
       </c>
-      <c r="U138" t="inlineStr">
+      <c r="X138" t="inlineStr">
         <is>
           <t>68822</t>
         </is>
@@ -8501,7 +8531,7 @@
           <t>NICHOLAS Jane</t>
         </is>
       </c>
-      <c r="U139" t="inlineStr">
+      <c r="X139" t="inlineStr">
         <is>
           <t>93757</t>
         </is>
@@ -8559,7 +8589,7 @@
           <t>THOMAS Hannah</t>
         </is>
       </c>
-      <c r="U140" t="inlineStr">
+      <c r="X140" t="inlineStr">
         <is>
           <t>85758</t>
         </is>
@@ -8617,7 +8647,7 @@
           <t>XU Yanru</t>
         </is>
       </c>
-      <c r="U141" t="inlineStr">
+      <c r="X141" t="inlineStr">
         <is>
           <t>63801</t>
         </is>
@@ -8675,7 +8705,7 @@
           <t>OTTEN Maartje</t>
         </is>
       </c>
-      <c r="U142" t="inlineStr">
+      <c r="X142" t="inlineStr">
         <is>
           <t>35337</t>
         </is>
@@ -8733,7 +8763,7 @@
           <t>RANDLE Kensa</t>
         </is>
       </c>
-      <c r="U143" t="inlineStr">
+      <c r="X143" t="inlineStr">
         <is>
           <t>51859</t>
         </is>
@@ -8791,7 +8821,7 @@
           <t>BETTERIDGE Lois</t>
         </is>
       </c>
-      <c r="U144" t="inlineStr">
+      <c r="X144" t="inlineStr">
         <is>
           <t>60078</t>
         </is>
@@ -8849,7 +8879,7 @@
           <t>MITASIKOVA Monika</t>
         </is>
       </c>
-      <c r="U145" t="inlineStr">
+      <c r="X145" t="inlineStr">
         <is>
           <t>75445</t>
         </is>
@@ -8907,7 +8937,7 @@
           <t>DONNELLY Sage</t>
         </is>
       </c>
-      <c r="U146" t="inlineStr">
+      <c r="X146" t="inlineStr">
         <is>
           <t>60119</t>
         </is>
@@ -8965,7 +8995,7 @@
           <t>MINAZOVA Alsu</t>
         </is>
       </c>
-      <c r="U147" t="inlineStr">
+      <c r="X147" t="inlineStr">
         <is>
           <t>53314</t>
         </is>
@@ -9023,7 +9053,7 @@
           <t>NEE Ashley</t>
         </is>
       </c>
-      <c r="U148" t="inlineStr">
+      <c r="X148" t="inlineStr">
         <is>
           <t>36363</t>
         </is>
@@ -9081,7 +9111,7 @@
           <t>VILARRUBLA Nuria</t>
         </is>
       </c>
-      <c r="U149" t="inlineStr">
+      <c r="X149" t="inlineStr">
         <is>
           <t>35746</t>
         </is>
@@ -9139,7 +9169,7 @@
           <t>APEL Elena</t>
         </is>
       </c>
-      <c r="U150" t="inlineStr">
+      <c r="X150" t="inlineStr">
         <is>
           <t>51837</t>
         </is>
@@ -9197,7 +9227,7 @@
           <t>FOX Noemie</t>
         </is>
       </c>
-      <c r="U151" t="inlineStr">
+      <c r="X151" t="inlineStr">
         <is>
           <t>44812</t>
         </is>
@@ -9255,7 +9285,7 @@
           <t>NOVAK Ajda</t>
         </is>
       </c>
-      <c r="U152" t="inlineStr">
+      <c r="X152" t="inlineStr">
         <is>
           <t>39079</t>
         </is>
@@ -9313,7 +9343,7 @@
           <t>DORIA VILARRUBLA Monica</t>
         </is>
       </c>
-      <c r="U153" t="inlineStr">
+      <c r="X153" t="inlineStr">
         <is>
           <t>53051</t>
         </is>
@@ -9371,7 +9401,7 @@
           <t>LI Tong</t>
         </is>
       </c>
-      <c r="U154" t="inlineStr">
+      <c r="X154" t="inlineStr">
         <is>
           <t>52023</t>
         </is>
@@ -9429,7 +9459,7 @@
           <t>PEROVA Ekaterina</t>
         </is>
       </c>
-      <c r="U155" t="inlineStr">
+      <c r="X155" t="inlineStr">
         <is>
           <t>35131</t>
         </is>
@@ -9487,7 +9517,7 @@
           <t>HILGERTOVA Amalie</t>
         </is>
       </c>
-      <c r="U156" t="inlineStr">
+      <c r="X156" t="inlineStr">
         <is>
           <t>36113</t>
         </is>
@@ -9545,7 +9575,7 @@
           <t>LAFONT Marie-Zelia</t>
         </is>
       </c>
-      <c r="U157" t="inlineStr">
+      <c r="X157" t="inlineStr">
         <is>
           <t>35374</t>
         </is>
@@ -9603,7 +9633,7 @@
           <t>LAWRENCE Rosalyn</t>
         </is>
       </c>
-      <c r="U158" t="inlineStr">
+      <c r="X158" t="inlineStr">
         <is>
           <t>36531</t>
         </is>
@@ -9661,7 +9691,7 @@
           <t>BAUDU Lucie</t>
         </is>
       </c>
-      <c r="U159" t="inlineStr">
+      <c r="X159" t="inlineStr">
         <is>
           <t>35669</t>
         </is>
@@ -9719,7 +9749,7 @@
           <t>KHARITONOVA Marta</t>
         </is>
       </c>
-      <c r="U160" t="inlineStr">
+      <c r="X160" t="inlineStr">
         <is>
           <t>35257</t>
         </is>
@@ -9777,7 +9807,7 @@
           <t>PACIERPNIK Natalia</t>
         </is>
       </c>
-      <c r="U161" t="inlineStr">
+      <c r="X161" t="inlineStr">
         <is>
           <t>35077</t>
         </is>
@@ -9835,7 +9865,7 @@
           <t>FRANKLIN Mallory</t>
         </is>
       </c>
-      <c r="U162" t="inlineStr">
+      <c r="X162" t="inlineStr">
         <is>
           <t>35615</t>
         </is>
@@ -10100,7 +10130,7 @@
           <t>ZWOLINSKA Klaudia</t>
         </is>
       </c>
-      <c r="U167" t="inlineStr">
+      <c r="X167" t="inlineStr">
         <is>
           <t>42027</t>
         </is>
@@ -10158,7 +10188,7 @@
           <t>TENG Qianqian</t>
         </is>
       </c>
-      <c r="U168" t="inlineStr">
+      <c r="X168" t="inlineStr">
         <is>
           <t>94209</t>
         </is>
@@ -10216,7 +10246,7 @@
           <t>LYU Minzhen</t>
         </is>
       </c>
-      <c r="U169" t="inlineStr">
+      <c r="X169" t="inlineStr">
         <is>
           <t>75379</t>
         </is>
@@ -10274,7 +10304,7 @@
           <t>THOMAS Hannah</t>
         </is>
       </c>
-      <c r="U170" t="inlineStr">
+      <c r="X170" t="inlineStr">
         <is>
           <t>85758</t>
         </is>
@@ -10332,7 +10362,7 @@
           <t>MICOZZI Elena</t>
         </is>
       </c>
-      <c r="U171" t="inlineStr">
+      <c r="X171" t="inlineStr">
         <is>
           <t>84644</t>
         </is>
@@ -10390,7 +10420,7 @@
           <t>O'FERRALL Caoimhe</t>
         </is>
       </c>
-      <c r="U172" t="inlineStr">
+      <c r="X172" t="inlineStr">
         <is>
           <t>61007</t>
         </is>
@@ -10448,7 +10478,7 @@
           <t>BETTERIDGE Lois</t>
         </is>
       </c>
-      <c r="U173" t="inlineStr">
+      <c r="X173" t="inlineStr">
         <is>
           <t>60078</t>
         </is>
@@ -10506,7 +10536,7 @@
           <t>OGILVIE Sophie</t>
         </is>
       </c>
-      <c r="U174" t="inlineStr">
+      <c r="X174" t="inlineStr">
         <is>
           <t>53134</t>
         </is>
@@ -10564,7 +10594,7 @@
           <t>HOCEVAR Eva Alina</t>
         </is>
       </c>
-      <c r="U175" t="inlineStr">
+      <c r="X175" t="inlineStr">
         <is>
           <t>75533</t>
         </is>
@@ -10622,7 +10652,7 @@
           <t>BERTONCELLI Marta</t>
         </is>
       </c>
-      <c r="U176" t="inlineStr">
+      <c r="X176" t="inlineStr">
         <is>
           <t>71982</t>
         </is>
@@ -10680,7 +10710,7 @@
           <t>BORGHI Elena</t>
         </is>
       </c>
-      <c r="U177" t="inlineStr">
+      <c r="X177" t="inlineStr">
         <is>
           <t>75493</t>
         </is>
@@ -10738,7 +10768,7 @@
           <t>LUKNAROVA Emanuela</t>
         </is>
       </c>
-      <c r="U178" t="inlineStr">
+      <c r="X178" t="inlineStr">
         <is>
           <t>76973</t>
         </is>
@@ -10796,7 +10826,7 @@
           <t>SCHORNBERG Jasmin</t>
         </is>
       </c>
-      <c r="U179" t="inlineStr">
+      <c r="X179" t="inlineStr">
         <is>
           <t>35206</t>
         </is>
@@ -10854,7 +10884,7 @@
           <t>CHEN Shi</t>
         </is>
       </c>
-      <c r="U180" t="inlineStr">
+      <c r="X180" t="inlineStr">
         <is>
           <t>52027</t>
         </is>
@@ -10912,7 +10942,7 @@
           <t>HAVLICKOVA Katerina</t>
         </is>
       </c>
-      <c r="U181" t="inlineStr">
+      <c r="X181" t="inlineStr">
         <is>
           <t>35048</t>
         </is>
@@ -10970,7 +11000,7 @@
           <t>BIZJAK Nina</t>
         </is>
       </c>
-      <c r="U182" t="inlineStr">
+      <c r="X182" t="inlineStr">
         <is>
           <t>39984</t>
         </is>
@@ -11028,7 +11058,7 @@
           <t>KOZOROG Alja</t>
         </is>
       </c>
-      <c r="U183" t="inlineStr">
+      <c r="X183" t="inlineStr">
         <is>
           <t>39986</t>
         </is>
@@ -11086,7 +11116,7 @@
           <t>DONNELLY Sage</t>
         </is>
       </c>
-      <c r="U184" t="inlineStr">
+      <c r="X184" t="inlineStr">
         <is>
           <t>60119</t>
         </is>
@@ -11144,7 +11174,7 @@
           <t>RIHOVA Eva</t>
         </is>
       </c>
-      <c r="U185" t="inlineStr">
+      <c r="X185" t="inlineStr">
         <is>
           <t>51791</t>
         </is>
@@ -11202,7 +11232,7 @@
           <t>APEL Elena</t>
         </is>
       </c>
-      <c r="U186" t="inlineStr">
+      <c r="X186" t="inlineStr">
         <is>
           <t>51837</t>
         </is>
@@ -11260,7 +11290,7 @@
           <t>SKACHOVA Monika</t>
         </is>
       </c>
-      <c r="U187" t="inlineStr">
+      <c r="X187" t="inlineStr">
         <is>
           <t>53078</t>
         </is>
@@ -11318,7 +11348,7 @@
           <t>MINAZOVA Alsu</t>
         </is>
       </c>
-      <c r="U188" t="inlineStr">
+      <c r="X188" t="inlineStr">
         <is>
           <t>53314</t>
         </is>
@@ -11376,7 +11406,7 @@
           <t>DORIA VILARRUBLA Monica</t>
         </is>
       </c>
-      <c r="U189" t="inlineStr">
+      <c r="X189" t="inlineStr">
         <is>
           <t>53051</t>
         </is>
@@ -11434,7 +11464,7 @@
           <t>SABITOVA Zulfia</t>
         </is>
       </c>
-      <c r="U190" t="inlineStr">
+      <c r="X190" t="inlineStr">
         <is>
           <t>40572</t>
         </is>
@@ -11492,7 +11522,7 @@
           <t>STANOVSKA Sona</t>
         </is>
       </c>
-      <c r="U191" t="inlineStr">
+      <c r="X191" t="inlineStr">
         <is>
           <t>51647</t>
         </is>
@@ -11550,7 +11580,7 @@
           <t>MUKHGALEEVA Polina</t>
         </is>
       </c>
-      <c r="U192" t="inlineStr">
+      <c r="X192" t="inlineStr">
         <is>
           <t>35768</t>
         </is>
@@ -11608,7 +11638,7 @@
           <t>BAUDU Lucie</t>
         </is>
       </c>
-      <c r="U193" t="inlineStr">
+      <c r="X193" t="inlineStr">
         <is>
           <t>35669</t>
         </is>
@@ -11666,7 +11696,7 @@
           <t>OLAZABAL Klara</t>
         </is>
       </c>
-      <c r="U194" t="inlineStr">
+      <c r="X194" t="inlineStr">
         <is>
           <t>43985</t>
         </is>
@@ -11724,7 +11754,7 @@
           <t>HERZOG Andrea</t>
         </is>
       </c>
-      <c r="U195" t="inlineStr">
+      <c r="X195" t="inlineStr">
         <is>
           <t>55099</t>
         </is>
@@ -11782,7 +11812,7 @@
           <t>JACQUET Claire</t>
         </is>
       </c>
-      <c r="U196" t="inlineStr">
+      <c r="X196" t="inlineStr">
         <is>
           <t>35684</t>
         </is>
@@ -11840,7 +11870,7 @@
           <t>FOX Noemie</t>
         </is>
       </c>
-      <c r="U197" t="inlineStr">
+      <c r="X197" t="inlineStr">
         <is>
           <t>44812</t>
         </is>
@@ -11898,7 +11928,7 @@
           <t>JONES Luuka</t>
         </is>
       </c>
-      <c r="U198" t="inlineStr">
+      <c r="X198" t="inlineStr">
         <is>
           <t>36657</t>
         </is>
@@ -11956,7 +11986,7 @@
           <t>LAWRENCE Rosalyn</t>
         </is>
       </c>
-      <c r="U199" t="inlineStr">
+      <c r="X199" t="inlineStr">
         <is>
           <t>36531</t>
         </is>
@@ -12014,7 +12044,7 @@
           <t>WOLFFHARDT Viktoria</t>
         </is>
       </c>
-      <c r="U200" t="inlineStr">
+      <c r="X200" t="inlineStr">
         <is>
           <t>35303</t>
         </is>
@@ -12072,7 +12102,7 @@
           <t>FISEROVA Tereza</t>
         </is>
       </c>
-      <c r="U201" t="inlineStr">
+      <c r="X201" t="inlineStr">
         <is>
           <t>42016</t>
         </is>
@@ -12130,7 +12160,7 @@
           <t>WOODS Kimberley</t>
         </is>
       </c>
-      <c r="U202" t="inlineStr">
+      <c r="X202" t="inlineStr">
         <is>
           <t>35650</t>
         </is>
@@ -12188,7 +12218,7 @@
           <t>SATILA Ana</t>
         </is>
       </c>
-      <c r="U203" t="inlineStr">
+      <c r="X203" t="inlineStr">
         <is>
           <t>35327</t>
         </is>
@@ -12246,7 +12276,7 @@
           <t>VILARRUBLA Nuria</t>
         </is>
       </c>
-      <c r="U204" t="inlineStr">
+      <c r="X204" t="inlineStr">
         <is>
           <t>35746</t>
         </is>
@@ -12304,7 +12334,7 @@
           <t>FRANKLIN Mallory</t>
         </is>
       </c>
-      <c r="U205" t="inlineStr">
+      <c r="X205" t="inlineStr">
         <is>
           <t>35615</t>
         </is>
@@ -12362,7 +12392,7 @@
           <t>FOX Jessica</t>
         </is>
       </c>
-      <c r="U206" t="inlineStr">
+      <c r="X206" t="inlineStr">
         <is>
           <t>36526</t>
         </is>
@@ -12420,7 +12450,7 @@
           <t>BOURHIS Yves</t>
         </is>
       </c>
-      <c r="U207" t="inlineStr">
+      <c r="X207" t="inlineStr">
         <is>
           <t>63237</t>
         </is>
@@ -12478,7 +12508,7 @@
           <t>ONG Jun Yi</t>
         </is>
       </c>
-      <c r="U208" t="inlineStr">
+      <c r="X208" t="inlineStr">
         <is>
           <t>75421</t>
         </is>
@@ -12536,7 +12566,7 @@
           <t>KOJIMA Daichi</t>
         </is>
       </c>
-      <c r="U209" t="inlineStr">
+      <c r="X209" t="inlineStr">
         <is>
           <t>42255</t>
         </is>
@@ -12594,7 +12624,7 @@
           <t>DESNOS Mathieu</t>
         </is>
       </c>
-      <c r="U210" t="inlineStr">
+      <c r="X210" t="inlineStr">
         <is>
           <t>93791</t>
         </is>
@@ -12652,7 +12682,7 @@
           <t>MUTO Yusuke</t>
         </is>
       </c>
-      <c r="U211" t="inlineStr">
+      <c r="X211" t="inlineStr">
         <is>
           <t>71820</t>
         </is>
@@ -12710,7 +12740,7 @@
           <t>FARRELL Oisin</t>
         </is>
       </c>
-      <c r="U212" t="inlineStr">
+      <c r="X212" t="inlineStr">
         <is>
           <t>37916</t>
         </is>
@@ -12768,7 +12798,7 @@
           <t>TEAGUE Eoin</t>
         </is>
       </c>
-      <c r="U213" t="inlineStr">
+      <c r="X213" t="inlineStr">
         <is>
           <t>37913</t>
         </is>
@@ -12826,7 +12856,7 @@
           <t>KARLSSON Max</t>
         </is>
       </c>
-      <c r="U214" t="inlineStr">
+      <c r="X214" t="inlineStr">
         <is>
           <t>35111</t>
         </is>
@@ -12884,7 +12914,7 @@
           <t>CURTIS Samuel</t>
         </is>
       </c>
-      <c r="U215" t="inlineStr">
+      <c r="X215" t="inlineStr">
         <is>
           <t>36683</t>
         </is>
@@ -12942,7 +12972,7 @@
           <t>KORPES Ren</t>
         </is>
       </c>
-      <c r="U216" t="inlineStr">
+      <c r="X216" t="inlineStr">
         <is>
           <t>39941</t>
         </is>
@@ -13000,7 +13030,7 @@
           <t>MAIMISTOV Sergey</t>
         </is>
       </c>
-      <c r="U217" t="inlineStr">
+      <c r="X217" t="inlineStr">
         <is>
           <t>53267</t>
         </is>
@@ -13058,7 +13088,7 @@
           <t>GUBENKO Nikita</t>
         </is>
       </c>
-      <c r="U218" t="inlineStr">
+      <c r="X218" t="inlineStr">
         <is>
           <t>39130</t>
         </is>
@@ -13116,7 +13146,7 @@
           <t>WAHLEN Fredrik</t>
         </is>
       </c>
-      <c r="U219" t="inlineStr">
+      <c r="X219" t="inlineStr">
         <is>
           <t>35102</t>
         </is>
@@ -13174,7 +13204,7 @@
           <t>TAYLER Michael</t>
         </is>
       </c>
-      <c r="U220" t="inlineStr">
+      <c r="X220" t="inlineStr">
         <is>
           <t>36262</t>
         </is>
@@ -13232,7 +13262,7 @@
           <t>YOSHIDA Taku</t>
         </is>
       </c>
-      <c r="U221" t="inlineStr">
+      <c r="X221" t="inlineStr">
         <is>
           <t>41611</t>
         </is>
@@ -13290,7 +13320,7 @@
           <t>DANGEN Jack</t>
         </is>
       </c>
-      <c r="U222" t="inlineStr">
+      <c r="X222" t="inlineStr">
         <is>
           <t>51865</t>
         </is>
@@ -13348,7 +13378,7 @@
           <t>HAYWARD Ben</t>
         </is>
       </c>
-      <c r="U223" t="inlineStr">
+      <c r="X223" t="inlineStr">
         <is>
           <t>35539</t>
         </is>
@@ -13406,7 +13436,7 @@
           <t>SILVA Ivan</t>
         </is>
       </c>
-      <c r="U224" t="inlineStr">
+      <c r="X224" t="inlineStr">
         <is>
           <t>35482</t>
         </is>
@@ -13464,7 +13494,7 @@
           <t>MUNSCH Manuel</t>
         </is>
       </c>
-      <c r="U225" t="inlineStr">
+      <c r="X225" t="inlineStr">
         <is>
           <t>35631</t>
         </is>
@@ -13522,7 +13552,7 @@
           <t>PRIOUX Lucie</t>
         </is>
       </c>
-      <c r="U226" t="inlineStr">
+      <c r="X226" t="inlineStr">
         <is>
           <t>42984</t>
         </is>
@@ -13580,7 +13610,7 @@
           <t>DOBY Mathieu</t>
         </is>
       </c>
-      <c r="U227" t="inlineStr">
+      <c r="X227" t="inlineStr">
         <is>
           <t>35292</t>
         </is>
@@ -13638,7 +13668,7 @@
           <t>MAJERCZAK Krzysztof</t>
         </is>
       </c>
-      <c r="U228" t="inlineStr">
+      <c r="X228" t="inlineStr">
         <is>
           <t>53647</t>
         </is>
@@ -13696,7 +13726,7 @@
           <t>BUTCHER Finn</t>
         </is>
       </c>
-      <c r="U229" t="inlineStr">
+      <c r="X229" t="inlineStr">
         <is>
           <t>36663</t>
         </is>
@@ -13754,7 +13784,7 @@
           <t>GILBERT Callum</t>
         </is>
       </c>
-      <c r="U230" t="inlineStr">
+      <c r="X230" t="inlineStr">
         <is>
           <t>42090</t>
         </is>
@@ -13812,7 +13842,7 @@
           <t>DE DIONIGI Christian</t>
         </is>
       </c>
-      <c r="U231" t="inlineStr">
+      <c r="X231" t="inlineStr">
         <is>
           <t>43188</t>
         </is>
@@ -13870,7 +13900,7 @@
           <t>BURGI Quentin</t>
         </is>
       </c>
-      <c r="U232" t="inlineStr">
+      <c r="X232" t="inlineStr">
         <is>
           <t>41590</t>
         </is>
@@ -13928,7 +13958,7 @@
           <t>BOWERS Christopher</t>
         </is>
       </c>
-      <c r="U233" t="inlineStr">
+      <c r="X233" t="inlineStr">
         <is>
           <t>52010</t>
         </is>
@@ -13986,7 +14016,7 @@
           <t>MAXEINER Tim</t>
         </is>
       </c>
-      <c r="U234" t="inlineStr">
+      <c r="X234" t="inlineStr">
         <is>
           <t>35117</t>
         </is>
@@ -14044,7 +14074,7 @@
           <t>MALEK Andrej</t>
         </is>
       </c>
-      <c r="U235" t="inlineStr">
+      <c r="X235" t="inlineStr">
         <is>
           <t>39246</t>
         </is>
@@ -14102,7 +14132,7 @@
           <t>TESTEN Niko</t>
         </is>
       </c>
-      <c r="U236" t="inlineStr">
+      <c r="X236" t="inlineStr">
         <is>
           <t>39980</t>
         </is>
@@ -14160,7 +14190,7 @@
           <t>MADORE Mathurin</t>
         </is>
       </c>
-      <c r="U237" t="inlineStr">
+      <c r="X237" t="inlineStr">
         <is>
           <t>51994</t>
         </is>
@@ -14218,7 +14248,7 @@
           <t>SRABOTNIK Martin</t>
         </is>
       </c>
-      <c r="U238" t="inlineStr">
+      <c r="X238" t="inlineStr">
         <is>
           <t>39080</t>
         </is>
@@ -14276,7 +14306,7 @@
           <t>GONCALVES Pedro</t>
         </is>
       </c>
-      <c r="U239" t="inlineStr">
+      <c r="X239" t="inlineStr">
         <is>
           <t>38017</t>
         </is>
@@ -14334,7 +14364,7 @@
           <t>OHRSTROM Isak</t>
         </is>
       </c>
-      <c r="U240" t="inlineStr">
+      <c r="X240" t="inlineStr">
         <is>
           <t>35101</t>
         </is>
@@ -14392,7 +14422,7 @@
           <t>LAUNAY Antoine</t>
         </is>
       </c>
-      <c r="U241" t="inlineStr">
+      <c r="X241" t="inlineStr">
         <is>
           <t>68776</t>
         </is>
@@ -14450,7 +14480,7 @@
           <t>HALCIN Martin</t>
         </is>
       </c>
-      <c r="U242" t="inlineStr">
+      <c r="X242" t="inlineStr">
         <is>
           <t>35355</t>
         </is>
@@ -14508,7 +14538,7 @@
           <t>ANDERSON Timothy</t>
         </is>
       </c>
-      <c r="U243" t="inlineStr">
+      <c r="X243" t="inlineStr">
         <is>
           <t>38432</t>
         </is>
@@ -14566,7 +14596,7 @@
           <t>HERNANZ Samuel</t>
         </is>
       </c>
-      <c r="U244" t="inlineStr">
+      <c r="X244" t="inlineStr">
         <is>
           <t>35786</t>
         </is>
@@ -14624,7 +14654,7 @@
           <t>EIGEL Pavel</t>
         </is>
       </c>
-      <c r="U245" t="inlineStr">
+      <c r="X245" t="inlineStr">
         <is>
           <t>35458</t>
         </is>
@@ -14682,7 +14712,7 @@
           <t>SCHWEIKERT Fabian</t>
         </is>
       </c>
-      <c r="U246" t="inlineStr">
+      <c r="X246" t="inlineStr">
         <is>
           <t>38412</t>
         </is>
@@ -14740,7 +14770,7 @@
           <t>LLORENTE David</t>
         </is>
       </c>
-      <c r="U247" t="inlineStr">
+      <c r="X247" t="inlineStr">
         <is>
           <t>51850</t>
         </is>
@@ -14798,7 +14828,7 @@
           <t>WERRO Lukas</t>
         </is>
       </c>
-      <c r="U248" t="inlineStr">
+      <c r="X248" t="inlineStr">
         <is>
           <t>35347</t>
         </is>
@@ -14856,7 +14886,7 @@
           <t>FORBES-CRYANS Bradley</t>
         </is>
       </c>
-      <c r="U249" t="inlineStr">
+      <c r="X249" t="inlineStr">
         <is>
           <t>36513</t>
         </is>
@@ -14914,7 +14944,7 @@
           <t>IVALDI Zeno</t>
         </is>
       </c>
-      <c r="U250" t="inlineStr">
+      <c r="X250" t="inlineStr">
         <is>
           <t>35480</t>
         </is>
@@ -14972,7 +15002,7 @@
           <t>HRADILEK Vavrinec</t>
         </is>
       </c>
-      <c r="U251" t="inlineStr">
+      <c r="X251" t="inlineStr">
         <is>
           <t>35031</t>
         </is>
@@ -15030,7 +15060,7 @@
           <t>PASIUT Michal</t>
         </is>
       </c>
-      <c r="U252" t="inlineStr">
+      <c r="X252" t="inlineStr">
         <is>
           <t>35095</t>
         </is>
@@ -15088,7 +15118,7 @@
           <t>WATKINS Daniel</t>
         </is>
       </c>
-      <c r="U253" t="inlineStr">
+      <c r="X253" t="inlineStr">
         <is>
           <t>38430</t>
         </is>
@@ -15146,7 +15176,7 @@
           <t>CRESPO Joan</t>
         </is>
       </c>
-      <c r="U254" t="inlineStr">
+      <c r="X254" t="inlineStr">
         <is>
           <t>35749</t>
         </is>
@@ -15204,7 +15234,7 @@
           <t>DOUGOUD Martin</t>
         </is>
       </c>
-      <c r="U255" t="inlineStr">
+      <c r="X255" t="inlineStr">
         <is>
           <t>35426</t>
         </is>
@@ -15262,7 +15292,7 @@
           <t>GRIGAR Jakub</t>
         </is>
       </c>
-      <c r="U256" t="inlineStr">
+      <c r="X256" t="inlineStr">
         <is>
           <t>37284</t>
         </is>
@@ -15320,7 +15350,7 @@
           <t>SMOLEN Michal</t>
         </is>
       </c>
-      <c r="U257" t="inlineStr">
+      <c r="X257" t="inlineStr">
         <is>
           <t>36397</t>
         </is>
@@ -15378,7 +15408,7 @@
           <t>POPIELA Dariusz</t>
         </is>
       </c>
-      <c r="U258" t="inlineStr">
+      <c r="X258" t="inlineStr">
         <is>
           <t>35096</t>
         </is>
@@ -15436,7 +15466,7 @@
           <t>DE GENNARO Giovanni</t>
         </is>
       </c>
-      <c r="U259" t="inlineStr">
+      <c r="X259" t="inlineStr">
         <is>
           <t>35244</t>
         </is>
@@ -15494,7 +15524,7 @@
           <t>DELFOUR Lucien</t>
         </is>
       </c>
-      <c r="U260" t="inlineStr">
+      <c r="X260" t="inlineStr">
         <is>
           <t>36537</t>
         </is>
@@ -15552,7 +15582,7 @@
           <t>NEVEU Boris</t>
         </is>
       </c>
-      <c r="U261" t="inlineStr">
+      <c r="X261" t="inlineStr">
         <is>
           <t>35396</t>
         </is>
@@ -15610,7 +15640,7 @@
           <t>AIGNER Hannes</t>
         </is>
       </c>
-      <c r="U262" t="inlineStr">
+      <c r="X262" t="inlineStr">
         <is>
           <t>35115</t>
         </is>
@@ -15668,7 +15698,7 @@
           <t>CLARKE Joseph</t>
         </is>
       </c>
-      <c r="U263" t="inlineStr">
+      <c r="X263" t="inlineStr">
         <is>
           <t>35654</t>
         </is>
@@ -15726,7 +15756,7 @@
           <t>PRSKAVEC Jiri</t>
         </is>
       </c>
-      <c r="U264" t="inlineStr">
+      <c r="X264" t="inlineStr">
         <is>
           <t>35033</t>
         </is>
@@ -15784,7 +15814,7 @@
           <t>KAUZER Peter</t>
         </is>
       </c>
-      <c r="U265" t="inlineStr">
+      <c r="X265" t="inlineStr">
         <is>
           <t>35589</t>
         </is>
@@ -15842,7 +15872,7 @@
           <t>PRINDIS Vit</t>
         </is>
       </c>
-      <c r="U266" t="inlineStr">
+      <c r="X266" t="inlineStr">
         <is>
           <t>35065</t>
         </is>
@@ -15900,7 +15930,7 @@
           <t>SANTOS Luca</t>
         </is>
       </c>
-      <c r="U267" t="inlineStr">
+      <c r="X267" t="inlineStr">
         <is>
           <t>69115</t>
         </is>
@@ -15958,7 +15988,7 @@
           <t>ZWOLINSKA Klaudia</t>
         </is>
       </c>
-      <c r="U268" t="inlineStr">
+      <c r="X268" t="inlineStr">
         <is>
           <t>42027</t>
         </is>
@@ -16016,7 +16046,7 @@
           <t>TENG Qianqian</t>
         </is>
       </c>
-      <c r="U269" t="inlineStr">
+      <c r="X269" t="inlineStr">
         <is>
           <t>94209</t>
         </is>
@@ -16074,7 +16104,7 @@
           <t>LYU Minzhen</t>
         </is>
       </c>
-      <c r="U270" t="inlineStr">
+      <c r="X270" t="inlineStr">
         <is>
           <t>75379</t>
         </is>
@@ -16132,7 +16162,7 @@
           <t>THOMAS Hannah</t>
         </is>
       </c>
-      <c r="U271" t="inlineStr">
+      <c r="X271" t="inlineStr">
         <is>
           <t>85758</t>
         </is>
@@ -16190,7 +16220,7 @@
           <t>MICOZZI Elena</t>
         </is>
       </c>
-      <c r="U272" t="inlineStr">
+      <c r="X272" t="inlineStr">
         <is>
           <t>84644</t>
         </is>
@@ -16248,7 +16278,7 @@
           <t>O'FERRALL Caoimhe</t>
         </is>
       </c>
-      <c r="U273" t="inlineStr">
+      <c r="X273" t="inlineStr">
         <is>
           <t>61007</t>
         </is>
@@ -16306,7 +16336,7 @@
           <t>BETTERIDGE Lois</t>
         </is>
       </c>
-      <c r="U274" t="inlineStr">
+      <c r="X274" t="inlineStr">
         <is>
           <t>60078</t>
         </is>
@@ -16364,7 +16394,7 @@
           <t>BERTONCELLI Marta</t>
         </is>
       </c>
-      <c r="U275" t="inlineStr">
+      <c r="X275" t="inlineStr">
         <is>
           <t>71982</t>
         </is>
@@ -16422,7 +16452,7 @@
           <t>BORGHI Elena</t>
         </is>
       </c>
-      <c r="U276" t="inlineStr">
+      <c r="X276" t="inlineStr">
         <is>
           <t>75493</t>
         </is>
@@ -16480,7 +16510,7 @@
           <t>LUKNAROVA Emanuela</t>
         </is>
       </c>
-      <c r="U277" t="inlineStr">
+      <c r="X277" t="inlineStr">
         <is>
           <t>76973</t>
         </is>
@@ -16538,7 +16568,7 @@
           <t>SCHORNBERG Jasmin</t>
         </is>
       </c>
-      <c r="U278" t="inlineStr">
+      <c r="X278" t="inlineStr">
         <is>
           <t>35206</t>
         </is>
@@ -16596,7 +16626,7 @@
           <t>CHEN Shi</t>
         </is>
       </c>
-      <c r="U279" t="inlineStr">
+      <c r="X279" t="inlineStr">
         <is>
           <t>52027</t>
         </is>
@@ -16654,7 +16684,7 @@
           <t>HAVLICKOVA Katerina</t>
         </is>
       </c>
-      <c r="U280" t="inlineStr">
+      <c r="X280" t="inlineStr">
         <is>
           <t>35048</t>
         </is>
@@ -16712,7 +16742,7 @@
           <t>BIZJAK Nina</t>
         </is>
       </c>
-      <c r="U281" t="inlineStr">
+      <c r="X281" t="inlineStr">
         <is>
           <t>39984</t>
         </is>
@@ -16770,7 +16800,7 @@
           <t>DONNELLY Sage</t>
         </is>
       </c>
-      <c r="U282" t="inlineStr">
+      <c r="X282" t="inlineStr">
         <is>
           <t>60119</t>
         </is>
@@ -16828,7 +16858,7 @@
           <t>RIHOVA Eva</t>
         </is>
       </c>
-      <c r="U283" t="inlineStr">
+      <c r="X283" t="inlineStr">
         <is>
           <t>51791</t>
         </is>
@@ -16886,7 +16916,7 @@
           <t>SKACHOVA Monika</t>
         </is>
       </c>
-      <c r="U284" t="inlineStr">
+      <c r="X284" t="inlineStr">
         <is>
           <t>53078</t>
         </is>
@@ -16944,7 +16974,7 @@
           <t>DORIA VILARRUBLA Monica</t>
         </is>
       </c>
-      <c r="U285" t="inlineStr">
+      <c r="X285" t="inlineStr">
         <is>
           <t>53051</t>
         </is>
@@ -17002,7 +17032,7 @@
           <t>SABITOVA Zulfia</t>
         </is>
       </c>
-      <c r="U286" t="inlineStr">
+      <c r="X286" t="inlineStr">
         <is>
           <t>40572</t>
         </is>
@@ -17060,7 +17090,7 @@
           <t>PRIOUX Lucie</t>
         </is>
       </c>
-      <c r="U287" t="inlineStr">
+      <c r="X287" t="inlineStr">
         <is>
           <t>42984</t>
         </is>
@@ -17118,7 +17148,7 @@
           <t>LAWRENCE Rosalyn</t>
         </is>
       </c>
-      <c r="U288" t="inlineStr">
+      <c r="X288" t="inlineStr">
         <is>
           <t>36531</t>
         </is>
@@ -17176,7 +17206,7 @@
           <t>BOURHIS Yves</t>
         </is>
       </c>
-      <c r="U289" t="inlineStr">
+      <c r="X289" t="inlineStr">
         <is>
           <t>63237</t>
         </is>
@@ -17234,7 +17264,7 @@
           <t>ONG Jun Yi</t>
         </is>
       </c>
-      <c r="U290" t="inlineStr">
+      <c r="X290" t="inlineStr">
         <is>
           <t>75421</t>
         </is>
@@ -17292,7 +17322,7 @@
           <t>SANTOS Luca</t>
         </is>
       </c>
-      <c r="U291" t="inlineStr">
+      <c r="X291" t="inlineStr">
         <is>
           <t>69115</t>
         </is>
@@ -17350,7 +17380,7 @@
           <t>KOJIMA Daichi</t>
         </is>
       </c>
-      <c r="U292" t="inlineStr">
+      <c r="X292" t="inlineStr">
         <is>
           <t>42255</t>
         </is>
@@ -17408,7 +17438,7 @@
           <t>DESNOS Mathieu</t>
         </is>
       </c>
-      <c r="U293" t="inlineStr">
+      <c r="X293" t="inlineStr">
         <is>
           <t>93791</t>
         </is>
@@ -17466,7 +17496,7 @@
           <t>MUTO Yusuke</t>
         </is>
       </c>
-      <c r="U294" t="inlineStr">
+      <c r="X294" t="inlineStr">
         <is>
           <t>71820</t>
         </is>
@@ -17524,7 +17554,7 @@
           <t>FARRELL Oisin</t>
         </is>
       </c>
-      <c r="U295" t="inlineStr">
+      <c r="X295" t="inlineStr">
         <is>
           <t>37916</t>
         </is>
@@ -17582,7 +17612,7 @@
           <t>TEAGUE Eoin</t>
         </is>
       </c>
-      <c r="U296" t="inlineStr">
+      <c r="X296" t="inlineStr">
         <is>
           <t>37913</t>
         </is>
@@ -17640,7 +17670,7 @@
           <t>KARLSSON Max</t>
         </is>
       </c>
-      <c r="U297" t="inlineStr">
+      <c r="X297" t="inlineStr">
         <is>
           <t>35111</t>
         </is>
@@ -17698,7 +17728,7 @@
           <t>CURTIS Samuel</t>
         </is>
       </c>
-      <c r="U298" t="inlineStr">
+      <c r="X298" t="inlineStr">
         <is>
           <t>36683</t>
         </is>
@@ -17756,7 +17786,7 @@
           <t>KORPES Ren</t>
         </is>
       </c>
-      <c r="U299" t="inlineStr">
+      <c r="X299" t="inlineStr">
         <is>
           <t>39941</t>
         </is>
@@ -17814,7 +17844,7 @@
           <t>MAIMISTOV Sergey</t>
         </is>
       </c>
-      <c r="U300" t="inlineStr">
+      <c r="X300" t="inlineStr">
         <is>
           <t>53267</t>
         </is>
@@ -17872,7 +17902,7 @@
           <t>GUBENKO Nikita</t>
         </is>
       </c>
-      <c r="U301" t="inlineStr">
+      <c r="X301" t="inlineStr">
         <is>
           <t>39130</t>
         </is>
@@ -17930,7 +17960,7 @@
           <t>WAHLEN Fredrik</t>
         </is>
       </c>
-      <c r="U302" t="inlineStr">
+      <c r="X302" t="inlineStr">
         <is>
           <t>35102</t>
         </is>
@@ -17988,7 +18018,7 @@
           <t>TAYLER Michael</t>
         </is>
       </c>
-      <c r="U303" t="inlineStr">
+      <c r="X303" t="inlineStr">
         <is>
           <t>36262</t>
         </is>
@@ -18046,7 +18076,7 @@
           <t>YOSHIDA Taku</t>
         </is>
       </c>
-      <c r="U304" t="inlineStr">
+      <c r="X304" t="inlineStr">
         <is>
           <t>41611</t>
         </is>
@@ -18104,7 +18134,7 @@
           <t>DANGEN Jack</t>
         </is>
       </c>
-      <c r="U305" t="inlineStr">
+      <c r="X305" t="inlineStr">
         <is>
           <t>51865</t>
         </is>
@@ -18162,7 +18192,7 @@
           <t>HAYWARD Ben</t>
         </is>
       </c>
-      <c r="U306" t="inlineStr">
+      <c r="X306" t="inlineStr">
         <is>
           <t>35539</t>
         </is>
@@ -18220,7 +18250,7 @@
           <t>SILVA Ivan</t>
         </is>
       </c>
-      <c r="U307" t="inlineStr">
+      <c r="X307" t="inlineStr">
         <is>
           <t>35482</t>
         </is>
@@ -18278,7 +18308,7 @@
           <t>MUNSCH Manuel</t>
         </is>
       </c>
-      <c r="U308" t="inlineStr">
+      <c r="X308" t="inlineStr">
         <is>
           <t>35631</t>
         </is>
@@ -18336,7 +18366,7 @@
           <t>DE DIONIGI Christian</t>
         </is>
       </c>
-      <c r="U309" t="inlineStr">
+      <c r="X309" t="inlineStr">
         <is>
           <t>43188</t>
         </is>
@@ -18394,7 +18424,7 @@
           <t>MALEK Andrej</t>
         </is>
       </c>
-      <c r="U310" t="inlineStr">
+      <c r="X310" t="inlineStr">
         <is>
           <t>39246</t>
         </is>
@@ -18452,7 +18482,7 @@
           <t>GONCALVES Pedro</t>
         </is>
       </c>
-      <c r="U311" t="inlineStr">
+      <c r="X311" t="inlineStr">
         <is>
           <t>38017</t>
         </is>
@@ -18510,7 +18540,7 @@
           <t>OHRSTROM Isak</t>
         </is>
       </c>
-      <c r="U312" t="inlineStr">
+      <c r="X312" t="inlineStr">
         <is>
           <t>35101</t>
         </is>
@@ -18568,7 +18598,7 @@
           <t>HERNANZ Samuel</t>
         </is>
       </c>
-      <c r="U313" t="inlineStr">
+      <c r="X313" t="inlineStr">
         <is>
           <t>35786</t>
         </is>
@@ -18626,7 +18656,7 @@
           <t>EIGEL Pavel</t>
         </is>
       </c>
-      <c r="U314" t="inlineStr">
+      <c r="X314" t="inlineStr">
         <is>
           <t>35458</t>
         </is>
@@ -18684,7 +18714,7 @@
           <t>SCHWEIKERT Fabian</t>
         </is>
       </c>
-      <c r="U315" t="inlineStr">
+      <c r="X315" t="inlineStr">
         <is>
           <t>38412</t>
         </is>
@@ -18742,7 +18772,7 @@
           <t>CRESPO Joan</t>
         </is>
       </c>
-      <c r="U316" t="inlineStr">
+      <c r="X316" t="inlineStr">
         <is>
           <t>35749</t>
         </is>
@@ -18800,7 +18830,7 @@
           <t>POPIELA Dariusz</t>
         </is>
       </c>
-      <c r="U317" t="inlineStr">
+      <c r="X317" t="inlineStr">
         <is>
           <t>35096</t>
         </is>
@@ -18858,7 +18888,7 @@
           <t>PRSKAVEC Jiri</t>
         </is>
       </c>
-      <c r="U318" t="inlineStr">
+      <c r="X318" t="inlineStr">
         <is>
           <t>35033</t>
         </is>
@@ -19487,7 +19517,7 @@
           <t>SZTUBA Igor</t>
         </is>
       </c>
-      <c r="U331" t="inlineStr">
+      <c r="X331" t="inlineStr">
         <is>
           <t>35087</t>
         </is>
@@ -19545,7 +19575,7 @@
           <t>JEGOU Liam</t>
         </is>
       </c>
-      <c r="U332" t="inlineStr">
+      <c r="X332" t="inlineStr">
         <is>
           <t>35820</t>
         </is>
@@ -19603,7 +19633,7 @@
           <t>IVALDI Raffaello</t>
         </is>
       </c>
-      <c r="U333" t="inlineStr">
+      <c r="X333" t="inlineStr">
         <is>
           <t>35227</t>
         </is>
@@ -19661,7 +19691,7 @@
           <t>HEGER Vojtech</t>
         </is>
       </c>
-      <c r="U334" t="inlineStr">
+      <c r="X334" t="inlineStr">
         <is>
           <t>68872</t>
         </is>
@@ -19719,7 +19749,7 @@
           <t>WATKINS Daniel</t>
         </is>
       </c>
-      <c r="U335" t="inlineStr">
+      <c r="X335" t="inlineStr">
         <is>
           <t>38430</t>
         </is>
@@ -19777,7 +19807,7 @@
           <t>BORROWS Ian</t>
         </is>
       </c>
-      <c r="U336" t="inlineStr">
+      <c r="X336" t="inlineStr">
         <is>
           <t>36534</t>
         </is>
@@ -19835,7 +19865,7 @@
           <t>EICHFELD Casey</t>
         </is>
       </c>
-      <c r="U337" t="inlineStr">
+      <c r="X337" t="inlineStr">
         <is>
           <t>35067</t>
         </is>
@@ -19893,7 +19923,7 @@
           <t>RAK Tomas</t>
         </is>
       </c>
-      <c r="U338" t="inlineStr">
+      <c r="X338" t="inlineStr">
         <is>
           <t>35056</t>
         </is>
@@ -19951,7 +19981,7 @@
           <t>JOLY Cedric</t>
         </is>
       </c>
-      <c r="U339" t="inlineStr">
+      <c r="X339" t="inlineStr">
         <is>
           <t>35681</t>
         </is>
@@ -20009,7 +20039,7 @@
           <t>HEDWIG Grzegorz</t>
         </is>
       </c>
-      <c r="U340" t="inlineStr">
+      <c r="X340" t="inlineStr">
         <is>
           <t>35465</t>
         </is>
@@ -20067,7 +20097,7 @@
           <t>BOURHIS Jean Pierre</t>
         </is>
       </c>
-      <c r="U341" t="inlineStr">
+      <c r="X341" t="inlineStr">
         <is>
           <t>36968</t>
         </is>
@@ -20125,7 +20155,7 @@
           <t>KOECHLIN Thomas</t>
         </is>
       </c>
-      <c r="U342" t="inlineStr">
+      <c r="X342" t="inlineStr">
         <is>
           <t>35419</t>
         </is>
@@ -20183,7 +20213,7 @@
           <t>WESTLEY Ryan</t>
         </is>
       </c>
-      <c r="U343" t="inlineStr">
+      <c r="X343" t="inlineStr">
         <is>
           <t>35651</t>
         </is>
@@ -20241,7 +20271,7 @@
           <t>SETKIN Kirill</t>
         </is>
       </c>
-      <c r="U344" t="inlineStr">
+      <c r="X344" t="inlineStr">
         <is>
           <t>35457</t>
         </is>
@@ -20299,7 +20329,7 @@
           <t>COLAZINGARI Roberto</t>
         </is>
       </c>
-      <c r="U345" t="inlineStr">
+      <c r="X345" t="inlineStr">
         <is>
           <t>35223</t>
         </is>
@@ -20357,7 +20387,7 @@
           <t>ROHAN Lukas</t>
         </is>
       </c>
-      <c r="U346" t="inlineStr">
+      <c r="X346" t="inlineStr">
         <is>
           <t>36114</t>
         </is>
@@ -20415,7 +20445,7 @@
           <t>SMEDLEY Cameron</t>
         </is>
       </c>
-      <c r="U347" t="inlineStr">
+      <c r="X347" t="inlineStr">
         <is>
           <t>35543</t>
         </is>
@@ -20473,7 +20503,7 @@
           <t>SZTUBA Kacper</t>
         </is>
       </c>
-      <c r="U348" t="inlineStr">
+      <c r="X348" t="inlineStr">
         <is>
           <t>53636</t>
         </is>
@@ -20531,7 +20561,7 @@
           <t>MARTIKAN Michal</t>
         </is>
       </c>
-      <c r="U349" t="inlineStr">
+      <c r="X349" t="inlineStr">
         <is>
           <t>35365</t>
         </is>
@@ -20589,7 +20619,7 @@
           <t>GARGAUD CHANUT Denis</t>
         </is>
       </c>
-      <c r="U350" t="inlineStr">
+      <c r="X350" t="inlineStr">
         <is>
           <t>35177</t>
         </is>
@@ -20647,7 +20677,7 @@
           <t>ELOSEGI Ander</t>
         </is>
       </c>
-      <c r="U351" t="inlineStr">
+      <c r="X351" t="inlineStr">
         <is>
           <t>35785</t>
         </is>
@@ -20705,7 +20735,7 @@
           <t>TASIADIS Sideris</t>
         </is>
       </c>
-      <c r="U352" t="inlineStr">
+      <c r="X352" t="inlineStr">
         <is>
           <t>35135</t>
         </is>
@@ -20763,7 +20793,7 @@
           <t>BURGESS Adam</t>
         </is>
       </c>
-      <c r="U353" t="inlineStr">
+      <c r="X353" t="inlineStr">
         <is>
           <t>35647</t>
         </is>
@@ -20821,7 +20851,7 @@
           <t>SLAFKOVSKY Alexander</t>
         </is>
       </c>
-      <c r="U354" t="inlineStr">
+      <c r="X354" t="inlineStr">
         <is>
           <t>35129</t>
         </is>
@@ -20879,7 +20909,7 @@
           <t>ANTON Franz</t>
         </is>
       </c>
-      <c r="U355" t="inlineStr">
+      <c r="X355" t="inlineStr">
         <is>
           <t>35137</t>
         </is>
@@ -20937,7 +20967,7 @@
           <t>BOZIC Luka</t>
         </is>
       </c>
-      <c r="U356" t="inlineStr">
+      <c r="X356" t="inlineStr">
         <is>
           <t>36269</t>
         </is>
@@ -20995,7 +21025,7 @@
           <t>SAVSEK Benjamin</t>
         </is>
       </c>
-      <c r="U357" t="inlineStr">
+      <c r="X357" t="inlineStr">
         <is>
           <t>36218</t>
         </is>
@@ -21053,7 +21083,7 @@
           <t>BENUS Matej</t>
         </is>
       </c>
-      <c r="U358" t="inlineStr">
+      <c r="X358" t="inlineStr">
         <is>
           <t>35353</t>
         </is>
@@ -21111,7 +21141,7 @@
           <t>FLORENCE David</t>
         </is>
       </c>
-      <c r="U359" t="inlineStr">
+      <c r="X359" t="inlineStr">
         <is>
           <t>35634</t>
         </is>
@@ -21169,7 +21199,7 @@
           <t>THOMAS Martin</t>
         </is>
       </c>
-      <c r="U360" t="inlineStr">
+      <c r="X360" t="inlineStr">
         <is>
           <t>35412</t>
         </is>
@@ -21227,7 +21257,7 @@
           <t>LI Tong</t>
         </is>
       </c>
-      <c r="U361" t="inlineStr">
+      <c r="X361" t="inlineStr">
         <is>
           <t>52023</t>
         </is>
@@ -21285,7 +21315,7 @@
           <t>NOVAK Ajda</t>
         </is>
       </c>
-      <c r="U362" t="inlineStr">
+      <c r="X362" t="inlineStr">
         <is>
           <t>39079</t>
         </is>
@@ -21343,7 +21373,7 @@
           <t>APEL Elena</t>
         </is>
       </c>
-      <c r="U363" t="inlineStr">
+      <c r="X363" t="inlineStr">
         <is>
           <t>51837</t>
         </is>
@@ -21401,7 +21431,7 @@
           <t>VILARRUBLA Nuria</t>
         </is>
       </c>
-      <c r="U364" t="inlineStr">
+      <c r="X364" t="inlineStr">
         <is>
           <t>35746</t>
         </is>
@@ -21459,7 +21489,7 @@
           <t>LAFONT Marie-Zelia</t>
         </is>
       </c>
-      <c r="U365" t="inlineStr">
+      <c r="X365" t="inlineStr">
         <is>
           <t>35374</t>
         </is>
@@ -21517,7 +21547,7 @@
           <t>FOX Noemie</t>
         </is>
       </c>
-      <c r="U366" t="inlineStr">
+      <c r="X366" t="inlineStr">
         <is>
           <t>44812</t>
         </is>
@@ -21575,7 +21605,7 @@
           <t>LAWRENCE Rosalyn</t>
         </is>
       </c>
-      <c r="U367" t="inlineStr">
+      <c r="X367" t="inlineStr">
         <is>
           <t>36531</t>
         </is>
@@ -21633,7 +21663,7 @@
           <t>HILGERTOVA Amalie</t>
         </is>
       </c>
-      <c r="U368" t="inlineStr">
+      <c r="X368" t="inlineStr">
         <is>
           <t>36113</t>
         </is>
@@ -21691,7 +21721,7 @@
           <t>BAUDU Lucie</t>
         </is>
       </c>
-      <c r="U369" t="inlineStr">
+      <c r="X369" t="inlineStr">
         <is>
           <t>35669</t>
         </is>
@@ -21749,7 +21779,7 @@
           <t>FRANKLIN Mallory</t>
         </is>
       </c>
-      <c r="U370" t="inlineStr">
+      <c r="X370" t="inlineStr">
         <is>
           <t>35615</t>
         </is>
@@ -21807,7 +21837,7 @@
           <t>KALISKA Elena</t>
         </is>
       </c>
-      <c r="U371" t="inlineStr">
+      <c r="X371" t="inlineStr">
         <is>
           <t>35366</t>
         </is>
@@ -21865,7 +21895,7 @@
           <t>SCHORNBERG Jasmin</t>
         </is>
       </c>
-      <c r="U372" t="inlineStr">
+      <c r="X372" t="inlineStr">
         <is>
           <t>35206</t>
         </is>
@@ -21923,7 +21953,7 @@
           <t>PRIGENT Camille</t>
         </is>
       </c>
-      <c r="U373" t="inlineStr">
+      <c r="X373" t="inlineStr">
         <is>
           <t>41566</t>
         </is>
@@ -21981,7 +22011,7 @@
           <t>KUHNLE Corinna</t>
         </is>
       </c>
-      <c r="U374" t="inlineStr">
+      <c r="X374" t="inlineStr">
         <is>
           <t>35282</t>
         </is>
@@ -22039,7 +22069,7 @@
           <t>JONES Luuka</t>
         </is>
       </c>
-      <c r="U375" t="inlineStr">
+      <c r="X375" t="inlineStr">
         <is>
           <t>36657</t>
         </is>
@@ -22097,7 +22127,7 @@
           <t>MINTALOVA Eliska</t>
         </is>
       </c>
-      <c r="U376" t="inlineStr">
+      <c r="X376" t="inlineStr">
         <is>
           <t>56169</t>
         </is>
@@ -22155,7 +22185,7 @@
           <t>FOX Jessica</t>
         </is>
       </c>
-      <c r="U377" t="inlineStr">
+      <c r="X377" t="inlineStr">
         <is>
           <t>36526</t>
         </is>
@@ -22213,7 +22243,7 @@
           <t>KRAGELJ Ursa</t>
         </is>
       </c>
-      <c r="U378" t="inlineStr">
+      <c r="X378" t="inlineStr">
         <is>
           <t>36264</t>
         </is>
@@ -22271,7 +22301,7 @@
           <t>ZWOLINSKA Klaudia</t>
         </is>
       </c>
-      <c r="U379" t="inlineStr">
+      <c r="X379" t="inlineStr">
         <is>
           <t>42027</t>
         </is>
@@ -22329,7 +22359,7 @@
           <t>WOLFFHARDT Viktoria</t>
         </is>
       </c>
-      <c r="U380" t="inlineStr">
+      <c r="X380" t="inlineStr">
         <is>
           <t>35303</t>
         </is>
@@ -22387,7 +22417,7 @@
           <t>VOJTOVA Veronika</t>
         </is>
       </c>
-      <c r="U381" t="inlineStr">
+      <c r="X381" t="inlineStr">
         <is>
           <t>35945</t>
         </is>
@@ -22445,7 +22475,7 @@
           <t>TERCELJ Eva</t>
         </is>
       </c>
-      <c r="U382" t="inlineStr">
+      <c r="X382" t="inlineStr">
         <is>
           <t>36263</t>
         </is>
@@ -22503,7 +22533,7 @@
           <t>SATILA Ana</t>
         </is>
       </c>
-      <c r="U383" t="inlineStr">
+      <c r="X383" t="inlineStr">
         <is>
           <t>35327</t>
         </is>
@@ -22561,7 +22591,7 @@
           <t>DUKATOVA Jana</t>
         </is>
       </c>
-      <c r="U384" t="inlineStr">
+      <c r="X384" t="inlineStr">
         <is>
           <t>35354</t>
         </is>
@@ -22619,7 +22649,7 @@
           <t>PENNIE Fiona</t>
         </is>
       </c>
-      <c r="U385" t="inlineStr">
+      <c r="X385" t="inlineStr">
         <is>
           <t>35638</t>
         </is>
@@ -22677,7 +22707,7 @@
           <t>CHOURRAUT Maialen</t>
         </is>
       </c>
-      <c r="U386" t="inlineStr">
+      <c r="X386" t="inlineStr">
         <is>
           <t>35787</t>
         </is>
@@ -22735,7 +22765,7 @@
           <t>KUDEJOVA Katerina</t>
         </is>
       </c>
-      <c r="U387" t="inlineStr">
+      <c r="X387" t="inlineStr">
         <is>
           <t>35034</t>
         </is>
@@ -22793,7 +22823,7 @@
           <t>HORN Stefanie</t>
         </is>
       </c>
-      <c r="U388" t="inlineStr">
+      <c r="X388" t="inlineStr">
         <is>
           <t>38417</t>
         </is>
@@ -22851,7 +22881,7 @@
           <t>FUNK Ricarda</t>
         </is>
       </c>
-      <c r="U389" t="inlineStr">
+      <c r="X389" t="inlineStr">
         <is>
           <t>35122</t>
         </is>
@@ -22909,7 +22939,7 @@
           <t>WOODS Kimberley</t>
         </is>
       </c>
-      <c r="U390" t="inlineStr">
+      <c r="X390" t="inlineStr">
         <is>
           <t>35650</t>
         </is>
@@ -22977,7 +23007,7 @@
           <t>BENUS Matej</t>
         </is>
       </c>
-      <c r="U391" t="inlineStr">
+      <c r="X391" t="inlineStr">
         <is>
           <t>35353</t>
         </is>
@@ -23045,7 +23075,7 @@
           <t>THOMAS Martin</t>
         </is>
       </c>
-      <c r="U392" t="inlineStr">
+      <c r="X392" t="inlineStr">
         <is>
           <t>35412</t>
         </is>
@@ -23113,7 +23143,7 @@
           <t>SAVSEK Benjamin</t>
         </is>
       </c>
-      <c r="U393" t="inlineStr">
+      <c r="X393" t="inlineStr">
         <is>
           <t>36218</t>
         </is>
@@ -23181,7 +23211,7 @@
           <t>IVALDI Raffaello</t>
         </is>
       </c>
-      <c r="U394" t="inlineStr">
+      <c r="X394" t="inlineStr">
         <is>
           <t>35227</t>
         </is>
@@ -23249,7 +23279,7 @@
           <t>BOZIC Luka</t>
         </is>
       </c>
-      <c r="U395" t="inlineStr">
+      <c r="X395" t="inlineStr">
         <is>
           <t>36269</t>
         </is>
@@ -23317,7 +23347,7 @@
           <t>TASIADIS Sideris</t>
         </is>
       </c>
-      <c r="U396" t="inlineStr">
+      <c r="X396" t="inlineStr">
         <is>
           <t>35135</t>
         </is>
@@ -23385,7 +23415,7 @@
           <t>WESTLEY Ryan</t>
         </is>
       </c>
-      <c r="U397" t="inlineStr">
+      <c r="X397" t="inlineStr">
         <is>
           <t>35651</t>
         </is>
@@ -23453,7 +23483,7 @@
           <t>FLORENCE David</t>
         </is>
       </c>
-      <c r="U398" t="inlineStr">
+      <c r="X398" t="inlineStr">
         <is>
           <t>35634</t>
         </is>
@@ -23521,7 +23551,7 @@
           <t>BURGESS Adam</t>
         </is>
       </c>
-      <c r="U399" t="inlineStr">
+      <c r="X399" t="inlineStr">
         <is>
           <t>35647</t>
         </is>
@@ -23589,7 +23619,7 @@
           <t>ANTON Franz</t>
         </is>
       </c>
-      <c r="U400" t="inlineStr">
+      <c r="X400" t="inlineStr">
         <is>
           <t>35137</t>
         </is>
@@ -23657,7 +23687,7 @@
           <t>CHOURRAUT Maialen</t>
         </is>
       </c>
-      <c r="U401" t="inlineStr">
+      <c r="X401" t="inlineStr">
         <is>
           <t>35787</t>
         </is>
@@ -23725,7 +23755,7 @@
           <t>HILGERTOVA Amalie</t>
         </is>
       </c>
-      <c r="U402" t="inlineStr">
+      <c r="X402" t="inlineStr">
         <is>
           <t>36113</t>
         </is>
@@ -23793,7 +23823,7 @@
           <t>TERCELJ Eva</t>
         </is>
       </c>
-      <c r="U403" t="inlineStr">
+      <c r="X403" t="inlineStr">
         <is>
           <t>36263</t>
         </is>
@@ -23861,7 +23891,7 @@
           <t>MINTALOVA Eliska</t>
         </is>
       </c>
-      <c r="U404" t="inlineStr">
+      <c r="X404" t="inlineStr">
         <is>
           <t>56169</t>
         </is>
@@ -23929,7 +23959,7 @@
           <t>WOODS Kimberley</t>
         </is>
       </c>
-      <c r="U405" t="inlineStr">
+      <c r="X405" t="inlineStr">
         <is>
           <t>35650</t>
         </is>
@@ -23997,7 +24027,7 @@
           <t>ZWOLINSKA Klaudia</t>
         </is>
       </c>
-      <c r="U406" t="inlineStr">
+      <c r="X406" t="inlineStr">
         <is>
           <t>42027</t>
         </is>
@@ -24065,7 +24095,7 @@
           <t>HORN Stefanie</t>
         </is>
       </c>
-      <c r="U407" t="inlineStr">
+      <c r="X407" t="inlineStr">
         <is>
           <t>38417</t>
         </is>
@@ -24133,7 +24163,7 @@
           <t>FUNK Ricarda</t>
         </is>
       </c>
-      <c r="U408" t="inlineStr">
+      <c r="X408" t="inlineStr">
         <is>
           <t>35122</t>
         </is>
@@ -24201,7 +24231,7 @@
           <t>FOX Jessica</t>
         </is>
       </c>
-      <c r="U409" t="inlineStr">
+      <c r="X409" t="inlineStr">
         <is>
           <t>36526</t>
         </is>
@@ -24269,7 +24299,7 @@
           <t>FRANKLIN Mallory</t>
         </is>
       </c>
-      <c r="U410" t="inlineStr">
+      <c r="X410" t="inlineStr">
         <is>
           <t>35615</t>
         </is>
@@ -24448,7 +24478,7 @@
           <t>HILGERTOVA Amalie</t>
         </is>
       </c>
-      <c r="U413" t="inlineStr">
+      <c r="X413" t="inlineStr">
         <is>
           <t>36113</t>
         </is>
@@ -24511,7 +24541,7 @@
           <t>MINAZOVA Alsu</t>
         </is>
       </c>
-      <c r="U414" t="inlineStr">
+      <c r="X414" t="inlineStr">
         <is>
           <t>53314</t>
         </is>
@@ -24574,7 +24604,7 @@
           <t>MUKHGALEEVA Polina</t>
         </is>
       </c>
-      <c r="U415" t="inlineStr">
+      <c r="X415" t="inlineStr">
         <is>
           <t>35768</t>
         </is>
@@ -24637,7 +24667,7 @@
           <t>NEE Ashley</t>
         </is>
       </c>
-      <c r="U416" t="inlineStr">
+      <c r="X416" t="inlineStr">
         <is>
           <t>36363</t>
         </is>
@@ -24700,7 +24730,7 @@
           <t>DAVIES Emily</t>
         </is>
       </c>
-      <c r="U417" t="inlineStr">
+      <c r="X417" t="inlineStr">
         <is>
           <t>87371</t>
         </is>
@@ -24763,7 +24793,7 @@
           <t>DONNELLY Sage</t>
         </is>
       </c>
-      <c r="U418" t="inlineStr">
+      <c r="X418" t="inlineStr">
         <is>
           <t>60119</t>
         </is>
@@ -24826,7 +24856,7 @@
           <t>AKINYEMI Johnathan</t>
         </is>
       </c>
-      <c r="U419" t="inlineStr">
+      <c r="X419" t="inlineStr">
         <is>
           <t>36822</t>
         </is>
@@ -24889,7 +24919,7 @@
           <t>CHAPPELL Etienne</t>
         </is>
       </c>
-      <c r="U420" t="inlineStr">
+      <c r="X420" t="inlineStr">
         <is>
           <t>75833</t>
         </is>
@@ -24952,7 +24982,7 @@
           <t>LONG Tren</t>
         </is>
       </c>
-      <c r="U421" t="inlineStr">
+      <c r="X421" t="inlineStr">
         <is>
           <t>57124</t>
         </is>
@@ -25015,7 +25045,7 @@
           <t>WAHLEN Fredrik</t>
         </is>
       </c>
-      <c r="U422" t="inlineStr">
+      <c r="X422" t="inlineStr">
         <is>
           <t>35102</t>
         </is>
@@ -25078,7 +25108,7 @@
           <t>DANGEN Jack</t>
         </is>
       </c>
-      <c r="U423" t="inlineStr">
+      <c r="X423" t="inlineStr">
         <is>
           <t>51865</t>
         </is>
@@ -25141,7 +25171,7 @@
           <t>GUBENKO Nikita</t>
         </is>
       </c>
-      <c r="U424" t="inlineStr">
+      <c r="X424" t="inlineStr">
         <is>
           <t>39130</t>
         </is>
@@ -25204,7 +25234,7 @@
           <t>HRADILEK Vavrinec</t>
         </is>
       </c>
-      <c r="U425" t="inlineStr">
+      <c r="X425" t="inlineStr">
         <is>
           <t>35031</t>
         </is>
@@ -25267,7 +25297,7 @@
           <t>SARAMANDIF Terence</t>
         </is>
       </c>
-      <c r="U426" t="inlineStr">
+      <c r="X426" t="inlineStr">
         <is>
           <t>79340</t>
         </is>
@@ -25388,7 +25418,7 @@
           <t>GONCALVES Pedro</t>
         </is>
       </c>
-      <c r="U428" t="inlineStr">
+      <c r="X428" t="inlineStr">
         <is>
           <t>38017</t>
         </is>
@@ -25451,7 +25481,7 @@
           <t>KARLSSON Max</t>
         </is>
       </c>
-      <c r="U429" t="inlineStr">
+      <c r="X429" t="inlineStr">
         <is>
           <t>35111</t>
         </is>
@@ -25572,7 +25602,7 @@
           <t>DE DIONIGI Christian</t>
         </is>
       </c>
-      <c r="U431" t="inlineStr">
+      <c r="X431" t="inlineStr">
         <is>
           <t>43188</t>
         </is>
@@ -25635,7 +25665,7 @@
           <t>KORPES Ren</t>
         </is>
       </c>
-      <c r="U432" t="inlineStr">
+      <c r="X432" t="inlineStr">
         <is>
           <t>39941</t>
         </is>
@@ -25698,7 +25728,7 @@
           <t>MAIMISTOV Sergey</t>
         </is>
       </c>
-      <c r="U433" t="inlineStr">
+      <c r="X433" t="inlineStr">
         <is>
           <t>53267</t>
         </is>
@@ -25761,7 +25791,7 @@
           <t>WHITE Aaron</t>
         </is>
       </c>
-      <c r="U434" t="inlineStr">
+      <c r="X434" t="inlineStr">
         <is>
           <t>92304</t>
         </is>
@@ -25882,7 +25912,7 @@
           <t>HILGERTOVA Amalie</t>
         </is>
       </c>
-      <c r="U436" t="inlineStr">
+      <c r="X436" t="inlineStr">
         <is>
           <t>36113</t>
         </is>
@@ -25945,7 +25975,7 @@
           <t>MINAZOVA Alsu</t>
         </is>
       </c>
-      <c r="U437" t="inlineStr">
+      <c r="X437" t="inlineStr">
         <is>
           <t>53314</t>
         </is>
@@ -26066,7 +26096,7 @@
           <t>DAVIES Emily</t>
         </is>
       </c>
-      <c r="U439" t="inlineStr">
+      <c r="X439" t="inlineStr">
         <is>
           <t>87371</t>
         </is>
@@ -26129,7 +26159,7 @@
           <t>DONNELLY Sage</t>
         </is>
       </c>
-      <c r="U440" t="inlineStr">
+      <c r="X440" t="inlineStr">
         <is>
           <t>60119</t>
         </is>
@@ -26192,7 +26222,7 @@
           <t>MUKHGALEEVA Polina</t>
         </is>
       </c>
-      <c r="U441" t="inlineStr">
+      <c r="X441" t="inlineStr">
         <is>
           <t>35768</t>
         </is>
@@ -26255,7 +26285,7 @@
           <t>NEE Ashley</t>
         </is>
       </c>
-      <c r="U442" t="inlineStr">
+      <c r="X442" t="inlineStr">
         <is>
           <t>36363</t>
         </is>
@@ -26318,7 +26348,7 @@
           <t>CHAPPELL Etienne</t>
         </is>
       </c>
-      <c r="U443" t="inlineStr">
+      <c r="X443" t="inlineStr">
         <is>
           <t>75833</t>
         </is>
@@ -26381,7 +26411,7 @@
           <t>DANGEN Jack</t>
         </is>
       </c>
-      <c r="U444" t="inlineStr">
+      <c r="X444" t="inlineStr">
         <is>
           <t>51865</t>
         </is>
@@ -26444,7 +26474,7 @@
           <t>HRADILEK Vavrinec</t>
         </is>
       </c>
-      <c r="U445" t="inlineStr">
+      <c r="X445" t="inlineStr">
         <is>
           <t>35031</t>
         </is>
@@ -26507,7 +26537,7 @@
           <t>LONG Tren</t>
         </is>
       </c>
-      <c r="U446" t="inlineStr">
+      <c r="X446" t="inlineStr">
         <is>
           <t>57124</t>
         </is>
@@ -26570,7 +26600,7 @@
           <t>DE DIONIGI Christian</t>
         </is>
       </c>
-      <c r="U447" t="inlineStr">
+      <c r="X447" t="inlineStr">
         <is>
           <t>43188</t>
         </is>
@@ -26691,7 +26721,7 @@
           <t>KARLSSON Max</t>
         </is>
       </c>
-      <c r="U449" t="inlineStr">
+      <c r="X449" t="inlineStr">
         <is>
           <t>35111</t>
         </is>
@@ -26754,7 +26784,7 @@
           <t>MAIMISTOV Sergey</t>
         </is>
       </c>
-      <c r="U450" t="inlineStr">
+      <c r="X450" t="inlineStr">
         <is>
           <t>53267</t>
         </is>
@@ -26827,7 +26857,7 @@
           <t>HILGERTOVA Amalie</t>
         </is>
       </c>
-      <c r="U451" t="inlineStr">
+      <c r="X451" t="inlineStr">
         <is>
           <t>36113</t>
         </is>
@@ -26900,7 +26930,7 @@
           <t>MINAZOVA Alsu</t>
         </is>
       </c>
-      <c r="U452" t="inlineStr">
+      <c r="X452" t="inlineStr">
         <is>
           <t>53314</t>
         </is>
@@ -26973,7 +27003,7 @@
           <t>MUKHGALEEVA Polina</t>
         </is>
       </c>
-      <c r="U453" t="inlineStr">
+      <c r="X453" t="inlineStr">
         <is>
           <t>35768</t>
         </is>
@@ -27046,7 +27076,7 @@
           <t>NEE Ashley</t>
         </is>
       </c>
-      <c r="U454" t="inlineStr">
+      <c r="X454" t="inlineStr">
         <is>
           <t>36363</t>
         </is>
@@ -27119,7 +27149,7 @@
           <t>CHAPPELL Etienne</t>
         </is>
       </c>
-      <c r="U455" t="inlineStr">
+      <c r="X455" t="inlineStr">
         <is>
           <t>75833</t>
         </is>
@@ -27192,7 +27222,7 @@
           <t>DE DIONIGI Christian</t>
         </is>
       </c>
-      <c r="U456" t="inlineStr">
+      <c r="X456" t="inlineStr">
         <is>
           <t>43188</t>
         </is>
@@ -27255,7 +27285,7 @@
           <t>HRADILEK Vavrinec</t>
         </is>
       </c>
-      <c r="U457" t="inlineStr">
+      <c r="X457" t="inlineStr">
         <is>
           <t>35031</t>
         </is>
@@ -27328,7 +27358,7 @@
           <t>MAIMISTOV Sergey</t>
         </is>
       </c>
-      <c r="U458" t="inlineStr">
+      <c r="X458" t="inlineStr">
         <is>
           <t>53267</t>
         </is>
@@ -27593,7 +27623,7 @@
           <t>RIHOVA Eva</t>
         </is>
       </c>
-      <c r="U463" t="inlineStr">
+      <c r="X463" t="inlineStr">
         <is>
           <t>51791</t>
         </is>
@@ -27651,7 +27681,7 @@
           <t>LAWRENCE Rosalyn</t>
         </is>
       </c>
-      <c r="U464" t="inlineStr">
+      <c r="X464" t="inlineStr">
         <is>
           <t>36531</t>
         </is>
@@ -27709,7 +27739,7 @@
           <t>BETTERIDGE Lois</t>
         </is>
       </c>
-      <c r="U465" t="inlineStr">
+      <c r="X465" t="inlineStr">
         <is>
           <t>60078</t>
         </is>
@@ -27767,7 +27797,7 @@
           <t>BERTONCELLI Marta</t>
         </is>
       </c>
-      <c r="U466" t="inlineStr">
+      <c r="X466" t="inlineStr">
         <is>
           <t>71982</t>
         </is>
@@ -27825,7 +27855,7 @@
           <t>LUKNAROVA Emanuela</t>
         </is>
       </c>
-      <c r="U467" t="inlineStr">
+      <c r="X467" t="inlineStr">
         <is>
           <t>76973</t>
         </is>
@@ -27883,7 +27913,7 @@
           <t>HAVLICKOVA Katerina</t>
         </is>
       </c>
-      <c r="U468" t="inlineStr">
+      <c r="X468" t="inlineStr">
         <is>
           <t>35048</t>
         </is>
@@ -27941,7 +27971,7 @@
           <t>SABITOVA Zulfia</t>
         </is>
       </c>
-      <c r="U469" t="inlineStr">
+      <c r="X469" t="inlineStr">
         <is>
           <t>40572</t>
         </is>
@@ -27999,7 +28029,7 @@
           <t>CHEN Shi</t>
         </is>
       </c>
-      <c r="U470" t="inlineStr">
+      <c r="X470" t="inlineStr">
         <is>
           <t>52027</t>
         </is>
@@ -28057,7 +28087,7 @@
           <t>SKACHOVA Monika</t>
         </is>
       </c>
-      <c r="U471" t="inlineStr">
+      <c r="X471" t="inlineStr">
         <is>
           <t>53078</t>
         </is>
@@ -28115,7 +28145,7 @@
           <t>DORIA VILARRUBLA Monica</t>
         </is>
       </c>
-      <c r="U472" t="inlineStr">
+      <c r="X472" t="inlineStr">
         <is>
           <t>53051</t>
         </is>
@@ -28173,7 +28203,7 @@
           <t>MUKHGALEEVA Polina</t>
         </is>
       </c>
-      <c r="U473" t="inlineStr">
+      <c r="X473" t="inlineStr">
         <is>
           <t>35768</t>
         </is>
@@ -28231,7 +28261,7 @@
           <t>HOCEVAR Eva Alina</t>
         </is>
       </c>
-      <c r="U474" t="inlineStr">
+      <c r="X474" t="inlineStr">
         <is>
           <t>75533</t>
         </is>
@@ -28289,7 +28319,7 @@
           <t>JACQUET Claire</t>
         </is>
       </c>
-      <c r="U475" t="inlineStr">
+      <c r="X475" t="inlineStr">
         <is>
           <t>35684</t>
         </is>
@@ -28347,7 +28377,7 @@
           <t>OLAZABAL Klara</t>
         </is>
       </c>
-      <c r="U476" t="inlineStr">
+      <c r="X476" t="inlineStr">
         <is>
           <t>43985</t>
         </is>
@@ -28405,7 +28435,7 @@
           <t>MINAZOVA Alsu</t>
         </is>
       </c>
-      <c r="U477" t="inlineStr">
+      <c r="X477" t="inlineStr">
         <is>
           <t>53314</t>
         </is>
@@ -28463,7 +28493,7 @@
           <t>JONES Luuka</t>
         </is>
       </c>
-      <c r="U478" t="inlineStr">
+      <c r="X478" t="inlineStr">
         <is>
           <t>36657</t>
         </is>
@@ -28521,7 +28551,7 @@
           <t>KOZOROG Alja</t>
         </is>
       </c>
-      <c r="U479" t="inlineStr">
+      <c r="X479" t="inlineStr">
         <is>
           <t>39986</t>
         </is>
@@ -28579,7 +28609,7 @@
           <t>WOLFFHARDT Viktoria</t>
         </is>
       </c>
-      <c r="U480" t="inlineStr">
+      <c r="X480" t="inlineStr">
         <is>
           <t>35303</t>
         </is>
@@ -28637,7 +28667,7 @@
           <t>STANOVSKA Sona</t>
         </is>
       </c>
-      <c r="U481" t="inlineStr">
+      <c r="X481" t="inlineStr">
         <is>
           <t>51647</t>
         </is>
@@ -28695,7 +28725,7 @@
           <t>APEL Elena</t>
         </is>
       </c>
-      <c r="U482" t="inlineStr">
+      <c r="X482" t="inlineStr">
         <is>
           <t>51837</t>
         </is>
@@ -28753,7 +28783,7 @@
           <t>FISEROVA Tereza</t>
         </is>
       </c>
-      <c r="U483" t="inlineStr">
+      <c r="X483" t="inlineStr">
         <is>
           <t>42016</t>
         </is>
@@ -28811,7 +28841,7 @@
           <t>OGILVIE Sophie</t>
         </is>
       </c>
-      <c r="U484" t="inlineStr">
+      <c r="X484" t="inlineStr">
         <is>
           <t>53134</t>
         </is>
@@ -28869,7 +28899,7 @@
           <t>FOX Noemie</t>
         </is>
       </c>
-      <c r="U485" t="inlineStr">
+      <c r="X485" t="inlineStr">
         <is>
           <t>44812</t>
         </is>
@@ -28927,7 +28957,7 @@
           <t>FRANKLIN Mallory</t>
         </is>
       </c>
-      <c r="U486" t="inlineStr">
+      <c r="X486" t="inlineStr">
         <is>
           <t>35615</t>
         </is>
@@ -28985,7 +29015,7 @@
           <t>VILARRUBLA Nuria</t>
         </is>
       </c>
-      <c r="U487" t="inlineStr">
+      <c r="X487" t="inlineStr">
         <is>
           <t>35746</t>
         </is>
@@ -29043,7 +29073,7 @@
           <t>HERZOG Andrea</t>
         </is>
       </c>
-      <c r="U488" t="inlineStr">
+      <c r="X488" t="inlineStr">
         <is>
           <t>55099</t>
         </is>
@@ -29101,7 +29131,7 @@
           <t>WOODS Kimberley</t>
         </is>
       </c>
-      <c r="U489" t="inlineStr">
+      <c r="X489" t="inlineStr">
         <is>
           <t>35650</t>
         </is>
@@ -29159,7 +29189,7 @@
           <t>BAUDU Lucie</t>
         </is>
       </c>
-      <c r="U490" t="inlineStr">
+      <c r="X490" t="inlineStr">
         <is>
           <t>35669</t>
         </is>
@@ -29217,7 +29247,7 @@
           <t>SATILA Ana</t>
         </is>
       </c>
-      <c r="U491" t="inlineStr">
+      <c r="X491" t="inlineStr">
         <is>
           <t>35327</t>
         </is>
@@ -29275,7 +29305,7 @@
           <t>FOX Jessica</t>
         </is>
       </c>
-      <c r="U492" t="inlineStr">
+      <c r="X492" t="inlineStr">
         <is>
           <t>36526</t>
         </is>
@@ -29333,7 +29363,7 @@
           <t>OTTEN Maartje</t>
         </is>
       </c>
-      <c r="U493" t="inlineStr">
+      <c r="X493" t="inlineStr">
         <is>
           <t>35337</t>
         </is>
@@ -29391,7 +29421,7 @@
           <t>DESNOS Mathieu</t>
         </is>
       </c>
-      <c r="U494" t="inlineStr">
+      <c r="X494" t="inlineStr">
         <is>
           <t>93791</t>
         </is>
@@ -29449,7 +29479,7 @@
           <t>CRESPO Joan</t>
         </is>
       </c>
-      <c r="U495" t="inlineStr">
+      <c r="X495" t="inlineStr">
         <is>
           <t>35749</t>
         </is>
@@ -29507,7 +29537,7 @@
           <t>DE DIONIGI Christian</t>
         </is>
       </c>
-      <c r="U496" t="inlineStr">
+      <c r="X496" t="inlineStr">
         <is>
           <t>43188</t>
         </is>
@@ -29565,7 +29595,7 @@
           <t>HAYWARD Ben</t>
         </is>
       </c>
-      <c r="U497" t="inlineStr">
+      <c r="X497" t="inlineStr">
         <is>
           <t>35539</t>
         </is>
@@ -29623,7 +29653,7 @@
           <t>HERNANZ Samuel</t>
         </is>
       </c>
-      <c r="U498" t="inlineStr">
+      <c r="X498" t="inlineStr">
         <is>
           <t>35786</t>
         </is>
@@ -29681,7 +29711,7 @@
           <t>YOSHIDA Taku</t>
         </is>
       </c>
-      <c r="U499" t="inlineStr">
+      <c r="X499" t="inlineStr">
         <is>
           <t>41611</t>
         </is>
@@ -29739,7 +29769,7 @@
           <t>MALEK Andrej</t>
         </is>
       </c>
-      <c r="U500" t="inlineStr">
+      <c r="X500" t="inlineStr">
         <is>
           <t>39246</t>
         </is>
@@ -29797,7 +29827,7 @@
           <t>TAYLER Michael</t>
         </is>
       </c>
-      <c r="U501" t="inlineStr">
+      <c r="X501" t="inlineStr">
         <is>
           <t>36262</t>
         </is>
@@ -29855,7 +29885,7 @@
           <t>POPIELA Dariusz</t>
         </is>
       </c>
-      <c r="U502" t="inlineStr">
+      <c r="X502" t="inlineStr">
         <is>
           <t>35096</t>
         </is>
@@ -29913,7 +29943,7 @@
           <t>PRSKAVEC Jiri</t>
         </is>
       </c>
-      <c r="U503" t="inlineStr">
+      <c r="X503" t="inlineStr">
         <is>
           <t>35033</t>
         </is>
@@ -29971,7 +30001,7 @@
           <t>TESTEN Niko</t>
         </is>
       </c>
-      <c r="U504" t="inlineStr">
+      <c r="X504" t="inlineStr">
         <is>
           <t>39980</t>
         </is>
@@ -30029,7 +30059,7 @@
           <t>NEVEU Boris</t>
         </is>
       </c>
-      <c r="U505" t="inlineStr">
+      <c r="X505" t="inlineStr">
         <is>
           <t>35396</t>
         </is>
@@ -30087,7 +30117,7 @@
           <t>MAJERCZAK Krzysztof</t>
         </is>
       </c>
-      <c r="U506" t="inlineStr">
+      <c r="X506" t="inlineStr">
         <is>
           <t>53647</t>
         </is>
@@ -30145,7 +30175,7 @@
           <t>WERRO Lukas</t>
         </is>
       </c>
-      <c r="U507" t="inlineStr">
+      <c r="X507" t="inlineStr">
         <is>
           <t>35347</t>
         </is>
@@ -30203,7 +30233,7 @@
           <t>DOBY Mathieu</t>
         </is>
       </c>
-      <c r="U508" t="inlineStr">
+      <c r="X508" t="inlineStr">
         <is>
           <t>35292</t>
         </is>
@@ -30261,7 +30291,7 @@
           <t>DOUGOUD Martin</t>
         </is>
       </c>
-      <c r="U509" t="inlineStr">
+      <c r="X509" t="inlineStr">
         <is>
           <t>35426</t>
         </is>
@@ -30319,7 +30349,7 @@
           <t>KAUZER Peter</t>
         </is>
       </c>
-      <c r="U510" t="inlineStr">
+      <c r="X510" t="inlineStr">
         <is>
           <t>35589</t>
         </is>
@@ -30377,7 +30407,7 @@
           <t>WATKINS Daniel</t>
         </is>
       </c>
-      <c r="U511" t="inlineStr">
+      <c r="X511" t="inlineStr">
         <is>
           <t>38430</t>
         </is>
@@ -30435,7 +30465,7 @@
           <t>SRABOTNIK Martin</t>
         </is>
       </c>
-      <c r="U512" t="inlineStr">
+      <c r="X512" t="inlineStr">
         <is>
           <t>39080</t>
         </is>
@@ -30493,7 +30523,7 @@
           <t>IVALDI Zeno</t>
         </is>
       </c>
-      <c r="U513" t="inlineStr">
+      <c r="X513" t="inlineStr">
         <is>
           <t>35480</t>
         </is>
@@ -30551,7 +30581,7 @@
           <t>SMOLEN Michal</t>
         </is>
       </c>
-      <c r="U514" t="inlineStr">
+      <c r="X514" t="inlineStr">
         <is>
           <t>36397</t>
         </is>
@@ -30609,7 +30639,7 @@
           <t>AIGNER Hannes</t>
         </is>
       </c>
-      <c r="U515" t="inlineStr">
+      <c r="X515" t="inlineStr">
         <is>
           <t>35115</t>
         </is>
@@ -30667,7 +30697,7 @@
           <t>PRINDIS Vit</t>
         </is>
       </c>
-      <c r="U516" t="inlineStr">
+      <c r="X516" t="inlineStr">
         <is>
           <t>35065</t>
         </is>
@@ -30725,7 +30755,7 @@
           <t>HALCIN Martin</t>
         </is>
       </c>
-      <c r="U517" t="inlineStr">
+      <c r="X517" t="inlineStr">
         <is>
           <t>35355</t>
         </is>
@@ -30783,7 +30813,7 @@
           <t>LAUNAY Antoine</t>
         </is>
       </c>
-      <c r="U518" t="inlineStr">
+      <c r="X518" t="inlineStr">
         <is>
           <t>68776</t>
         </is>
@@ -30841,7 +30871,7 @@
           <t>DE GENNARO Giovanni</t>
         </is>
       </c>
-      <c r="U519" t="inlineStr">
+      <c r="X519" t="inlineStr">
         <is>
           <t>35244</t>
         </is>
@@ -30899,7 +30929,7 @@
           <t>ANDERSON Timothy</t>
         </is>
       </c>
-      <c r="U520" t="inlineStr">
+      <c r="X520" t="inlineStr">
         <is>
           <t>38432</t>
         </is>
@@ -30957,7 +30987,7 @@
           <t>MADORE Mathurin</t>
         </is>
       </c>
-      <c r="U521" t="inlineStr">
+      <c r="X521" t="inlineStr">
         <is>
           <t>51994</t>
         </is>
@@ -31015,7 +31045,7 @@
           <t>GILBERT Callum</t>
         </is>
       </c>
-      <c r="U522" t="inlineStr">
+      <c r="X522" t="inlineStr">
         <is>
           <t>42090</t>
         </is>
@@ -31073,7 +31103,7 @@
           <t>BUTCHER Finn</t>
         </is>
       </c>
-      <c r="U523" t="inlineStr">
+      <c r="X523" t="inlineStr">
         <is>
           <t>36663</t>
         </is>
@@ -31131,7 +31161,7 @@
           <t>PASIUT Michal</t>
         </is>
       </c>
-      <c r="U524" t="inlineStr">
+      <c r="X524" t="inlineStr">
         <is>
           <t>35095</t>
         </is>
@@ -31189,7 +31219,7 @@
           <t>LLORENTE David</t>
         </is>
       </c>
-      <c r="U525" t="inlineStr">
+      <c r="X525" t="inlineStr">
         <is>
           <t>51850</t>
         </is>
@@ -31247,7 +31277,7 @@
           <t>MAXEINER Tim</t>
         </is>
       </c>
-      <c r="U526" t="inlineStr">
+      <c r="X526" t="inlineStr">
         <is>
           <t>35117</t>
         </is>
@@ -31305,7 +31335,7 @@
           <t>GRIGAR Jakub</t>
         </is>
       </c>
-      <c r="U527" t="inlineStr">
+      <c r="X527" t="inlineStr">
         <is>
           <t>37284</t>
         </is>
@@ -31363,7 +31393,7 @@
           <t>HRADILEK Vavrinec</t>
         </is>
       </c>
-      <c r="U528" t="inlineStr">
+      <c r="X528" t="inlineStr">
         <is>
           <t>35031</t>
         </is>
@@ -31421,7 +31451,7 @@
           <t>DELFOUR Lucien</t>
         </is>
       </c>
-      <c r="U529" t="inlineStr">
+      <c r="X529" t="inlineStr">
         <is>
           <t>36537</t>
         </is>
@@ -31479,7 +31509,7 @@
           <t>BOWERS Christopher</t>
         </is>
       </c>
-      <c r="U530" t="inlineStr">
+      <c r="X530" t="inlineStr">
         <is>
           <t>52010</t>
         </is>
@@ -31537,7 +31567,7 @@
           <t>BURGI Quentin</t>
         </is>
       </c>
-      <c r="U531" t="inlineStr">
+      <c r="X531" t="inlineStr">
         <is>
           <t>41590</t>
         </is>
@@ -31595,7 +31625,7 @@
           <t>FORBES-CRYANS Bradley</t>
         </is>
       </c>
-      <c r="U532" t="inlineStr">
+      <c r="X532" t="inlineStr">
         <is>
           <t>36513</t>
         </is>
@@ -31653,7 +31683,7 @@
           <t>CLARKE Joseph</t>
         </is>
       </c>
-      <c r="U533" t="inlineStr">
+      <c r="X533" t="inlineStr">
         <is>
           <t>35654</t>
         </is>
@@ -31721,7 +31751,7 @@
           <t>OLAZABAL Klara</t>
         </is>
       </c>
-      <c r="U534" t="inlineStr">
+      <c r="X534" t="inlineStr">
         <is>
           <t>43985</t>
         </is>
@@ -31789,7 +31819,7 @@
           <t>MINAZOVA Alsu</t>
         </is>
       </c>
-      <c r="U535" t="inlineStr">
+      <c r="X535" t="inlineStr">
         <is>
           <t>53314</t>
         </is>
@@ -31857,7 +31887,7 @@
           <t>JACQUET Claire</t>
         </is>
       </c>
-      <c r="U536" t="inlineStr">
+      <c r="X536" t="inlineStr">
         <is>
           <t>35684</t>
         </is>
@@ -31925,7 +31955,7 @@
           <t>BAUDU Lucie</t>
         </is>
       </c>
-      <c r="U537" t="inlineStr">
+      <c r="X537" t="inlineStr">
         <is>
           <t>35669</t>
         </is>
@@ -31993,7 +32023,7 @@
           <t>WOODS Kimberley</t>
         </is>
       </c>
-      <c r="U538" t="inlineStr">
+      <c r="X538" t="inlineStr">
         <is>
           <t>35650</t>
         </is>
@@ -32061,7 +32091,7 @@
           <t>FISEROVA Tereza</t>
         </is>
       </c>
-      <c r="U539" t="inlineStr">
+      <c r="X539" t="inlineStr">
         <is>
           <t>42016</t>
         </is>
@@ -32129,7 +32159,7 @@
           <t>HERZOG Andrea</t>
         </is>
       </c>
-      <c r="U540" t="inlineStr">
+      <c r="X540" t="inlineStr">
         <is>
           <t>55099</t>
         </is>
@@ -32197,7 +32227,7 @@
           <t>OGILVIE Sophie</t>
         </is>
       </c>
-      <c r="U541" t="inlineStr">
+      <c r="X541" t="inlineStr">
         <is>
           <t>53134</t>
         </is>
@@ -32265,7 +32295,7 @@
           <t>FOX Jessica</t>
         </is>
       </c>
-      <c r="U542" t="inlineStr">
+      <c r="X542" t="inlineStr">
         <is>
           <t>36526</t>
         </is>
@@ -32333,7 +32363,7 @@
           <t>FRANKLIN Mallory</t>
         </is>
       </c>
-      <c r="U543" t="inlineStr">
+      <c r="X543" t="inlineStr">
         <is>
           <t>35615</t>
         </is>
@@ -32401,7 +32431,7 @@
           <t>AIGNER Hannes</t>
         </is>
       </c>
-      <c r="U544" t="inlineStr">
+      <c r="X544" t="inlineStr">
         <is>
           <t>35115</t>
         </is>
@@ -32469,7 +32499,7 @@
           <t>LLORENTE David</t>
         </is>
       </c>
-      <c r="U545" t="inlineStr">
+      <c r="X545" t="inlineStr">
         <is>
           <t>51850</t>
         </is>
@@ -32537,7 +32567,7 @@
           <t>TESTEN Niko</t>
         </is>
       </c>
-      <c r="U546" t="inlineStr">
+      <c r="X546" t="inlineStr">
         <is>
           <t>39980</t>
         </is>
@@ -32605,7 +32635,7 @@
           <t>BOWERS Christopher</t>
         </is>
       </c>
-      <c r="U547" t="inlineStr">
+      <c r="X547" t="inlineStr">
         <is>
           <t>52010</t>
         </is>
@@ -32673,7 +32703,7 @@
           <t>KAUZER Peter</t>
         </is>
       </c>
-      <c r="U548" t="inlineStr">
+      <c r="X548" t="inlineStr">
         <is>
           <t>35589</t>
         </is>
@@ -32741,7 +32771,7 @@
           <t>GILBERT Callum</t>
         </is>
       </c>
-      <c r="U549" t="inlineStr">
+      <c r="X549" t="inlineStr">
         <is>
           <t>42090</t>
         </is>
@@ -32809,7 +32839,7 @@
           <t>WATKINS Daniel</t>
         </is>
       </c>
-      <c r="U550" t="inlineStr">
+      <c r="X550" t="inlineStr">
         <is>
           <t>38430</t>
         </is>
@@ -32877,7 +32907,7 @@
           <t>PASIUT Michal</t>
         </is>
       </c>
-      <c r="U551" t="inlineStr">
+      <c r="X551" t="inlineStr">
         <is>
           <t>35095</t>
         </is>
@@ -32945,7 +32975,7 @@
           <t>PRSKAVEC Jiri</t>
         </is>
       </c>
-      <c r="U552" t="inlineStr">
+      <c r="X552" t="inlineStr">
         <is>
           <t>35033</t>
         </is>
@@ -33013,7 +33043,7 @@
           <t>CLARKE Joseph</t>
         </is>
       </c>
-      <c r="U553" t="inlineStr">
+      <c r="X553" t="inlineStr">
         <is>
           <t>35654</t>
         </is>
@@ -33076,7 +33106,7 @@
           <t>DAVIES Emily</t>
         </is>
       </c>
-      <c r="U554" t="inlineStr">
+      <c r="X554" t="inlineStr">
         <is>
           <t>87371</t>
         </is>
@@ -33139,7 +33169,7 @@
           <t>HILGERTOVA Amalie</t>
         </is>
       </c>
-      <c r="U555" t="inlineStr">
+      <c r="X555" t="inlineStr">
         <is>
           <t>36113</t>
         </is>
@@ -33260,7 +33290,7 @@
           <t>MUKHGALEEVA Polina</t>
         </is>
       </c>
-      <c r="U557" t="inlineStr">
+      <c r="X557" t="inlineStr">
         <is>
           <t>35768</t>
         </is>
@@ -33381,7 +33411,7 @@
           <t>DONNELLY Sage</t>
         </is>
       </c>
-      <c r="U559" t="inlineStr">
+      <c r="X559" t="inlineStr">
         <is>
           <t>60119</t>
         </is>
@@ -33444,7 +33474,7 @@
           <t>MINAZOVA Alsu</t>
         </is>
       </c>
-      <c r="U560" t="inlineStr">
+      <c r="X560" t="inlineStr">
         <is>
           <t>53314</t>
         </is>
@@ -33507,7 +33537,7 @@
           <t>NEE Ashley</t>
         </is>
       </c>
-      <c r="U561" t="inlineStr">
+      <c r="X561" t="inlineStr">
         <is>
           <t>36363</t>
         </is>
@@ -33570,7 +33600,7 @@
           <t>AKINYEMI Johnathan</t>
         </is>
       </c>
-      <c r="U562" t="inlineStr">
+      <c r="X562" t="inlineStr">
         <is>
           <t>36822</t>
         </is>
@@ -33633,7 +33663,7 @@
           <t>HAYWARD Ben</t>
         </is>
       </c>
-      <c r="U563" t="inlineStr">
+      <c r="X563" t="inlineStr">
         <is>
           <t>35539</t>
         </is>
@@ -33696,7 +33726,7 @@
           <t>HRADILEK Vavrinec</t>
         </is>
       </c>
-      <c r="U564" t="inlineStr">
+      <c r="X564" t="inlineStr">
         <is>
           <t>35031</t>
         </is>
@@ -33759,7 +33789,7 @@
           <t>DE DIONIGI Christian</t>
         </is>
       </c>
-      <c r="U565" t="inlineStr">
+      <c r="X565" t="inlineStr">
         <is>
           <t>43188</t>
         </is>
@@ -33822,7 +33852,7 @@
           <t>GUBENKO Nikita</t>
         </is>
       </c>
-      <c r="U566" t="inlineStr">
+      <c r="X566" t="inlineStr">
         <is>
           <t>39130</t>
         </is>
@@ -33885,7 +33915,7 @@
           <t>GONCALVES Pedro</t>
         </is>
       </c>
-      <c r="U567" t="inlineStr">
+      <c r="X567" t="inlineStr">
         <is>
           <t>38017</t>
         </is>
@@ -33948,7 +33978,7 @@
           <t>WHITE Aaron</t>
         </is>
       </c>
-      <c r="U568" t="inlineStr">
+      <c r="X568" t="inlineStr">
         <is>
           <t>92304</t>
         </is>
@@ -34011,7 +34041,7 @@
           <t>KORPES Ren</t>
         </is>
       </c>
-      <c r="U569" t="inlineStr">
+      <c r="X569" t="inlineStr">
         <is>
           <t>39941</t>
         </is>
@@ -34132,7 +34162,7 @@
           <t>LONG Tren</t>
         </is>
       </c>
-      <c r="U571" t="inlineStr">
+      <c r="X571" t="inlineStr">
         <is>
           <t>57124</t>
         </is>
@@ -34195,7 +34225,7 @@
           <t>DANGEN Jack</t>
         </is>
       </c>
-      <c r="U572" t="inlineStr">
+      <c r="X572" t="inlineStr">
         <is>
           <t>51865</t>
         </is>
@@ -34258,7 +34288,7 @@
           <t>KARLSSON Max</t>
         </is>
       </c>
-      <c r="U573" t="inlineStr">
+      <c r="X573" t="inlineStr">
         <is>
           <t>35111</t>
         </is>
@@ -34321,7 +34351,7 @@
           <t>MAIMISTOV Sergey</t>
         </is>
       </c>
-      <c r="U574" t="inlineStr">
+      <c r="X574" t="inlineStr">
         <is>
           <t>53267</t>
         </is>
@@ -34384,7 +34414,7 @@
           <t>SARAMANDIF Terence</t>
         </is>
       </c>
-      <c r="U575" t="inlineStr">
+      <c r="X575" t="inlineStr">
         <is>
           <t>79340</t>
         </is>
@@ -34505,7 +34535,7 @@
           <t>TAYLER Michael</t>
         </is>
       </c>
-      <c r="U577" t="inlineStr">
+      <c r="X577" t="inlineStr">
         <is>
           <t>36262</t>
         </is>
@@ -34568,7 +34598,7 @@
           <t>WAHLEN Fredrik</t>
         </is>
       </c>
-      <c r="U578" t="inlineStr">
+      <c r="X578" t="inlineStr">
         <is>
           <t>35102</t>
         </is>
@@ -34631,7 +34661,7 @@
           <t>CHAPPELL Etienne</t>
         </is>
       </c>
-      <c r="U579" t="inlineStr">
+      <c r="X579" t="inlineStr">
         <is>
           <t>75833</t>
         </is>

</xml_diff>